<commit_message>
feat: goal profile compiler - convert natural language to structured JSON, reuse across searches to save AI tokens
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2342,11 +2342,763 @@
           <t>https://youtube.com/watch?v=02V_bAxmxfc</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Global dialogue on artificial intelligence governance - Opening session</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Watch the plenary presentation of the annual report of the multidisciplinary Independent International Scientific Panel on Artificial ...</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>2026-07-06T07:10:36Z</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=s_q3TU6ZKUk</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>No Holds Barred Radio Automation</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>2026-06-29T04:02:01Z</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=EzhSAzTqKtM</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>【FGU 4KLiveCam｜GenAI LiveChat】佛光大學＠蘭陽平原 即時影像 Lanyang Plain Live View</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>即時鳥瞰  美景共享× GenAI即時景色聊聊  ｜ 佛光大學正式啟用「即時影像網路直播」！  ✨ 坐落於礁溪林美山上的佛大，透過網 ...</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>2026-07-06T07:30:31Z</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=GS0p1OoeoDM</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>XonoBots — Professional Tools for YouTube &amp;amp; Twitch Creators | Grow Faster with Automation</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>XonoBots — Professional Tools for YouTube and Twitch Creators Take your content to the next level with XonoBots, a powerful ...</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>2026-02-12T07:00:00Z</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=5N22-QgCFqY</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Live Stream Bot Automation Tool | 유튜브 채널 자동 성장 봇</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>This video introduces a powerful Live Stream Automation Bot designed to help creators manage chat activity, comments, likes, ...</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>2026-02-14T07:30:00Z</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=xk8efUPDXXU</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>What Is AI ? | Learning Videos For Kids | Artificial Intelligence Explained | EMoMee</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Hello Curious Kids! In today's fun cartoon, we dive into one of those big “WHY?” questions curious kids like you love to ask!</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>2026-06-02T09:57:27Z</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=hs67716TQ3U</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>LIVE: Opening Session of Global Dialogue on Artificial Intelligence Governance | Day 1</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>The Global Dialogue on Artificial Intelligence Governance begins with its Day 1 Opening Session, bringing together government ...</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2026-07-06T09:15:24Z</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=l-N7mbtTtaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Automate With Python| Live Code |  AI Engineer | Back to Basics After AI Layoff 2026 |</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Learn Data Engineering from scratch with practical examples, real-world projects, and industry best practices. In this video, you'll ...</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>2026-07-06T07:30:20Z</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=dpwt9QmVYLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>How To Get Watching &amp;amp; Likes, Chats in Live Streams &amp;amp; Grow With Pbh STORE Softwares With Mobile Or PC</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>How To Get Watching &amp; Likes, Chats in Live Streams &amp; Grow With Pbh STORE Softwares With Mobile Or PC #Bot #StreamBot ...</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>2026-02-12T05:40:00Z</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=9-mmDf7FBX4</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Inside Modern Factory: How Plantain Chips Are Processed | Full Production Line (24/7 LIVE)</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Welcome to AGRO FACTORY SECRETS — your ultimate destination for discovering how everyday foods are processed inside ...</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2026-04-17T16:10:00Z</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=A6ifA-SUfm8</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>YouTube Live View Bot ❤️‍🔥YOUTUBE VIEW BOT | LIVE Growth Tool Demo — Increase Likes, Subs &amp;amp; Comments</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Welcome to the LIVE demo of XONO Bots — Live Stream Automation Software This stream shows how you can manage ...</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>2026-04-20T09:15:00Z</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=JMd-1ikizdA</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Turn $100 into $1,000,000 Challenge with Trading Bot 🔥 MT4 Real Account ( FREE EA )</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Trading Bot Challenge (LIVE) What if you could turn a small account into something massive… using pure automation? In this live ...</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>2026-06-29T04:42:59Z</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=VhAL5PoisiE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>YBE AI – Your All-in-One Free AI Platform 🇮🇳</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Link ai.ybeapp.com **Welcome to YBE AI – Your All-in-One Free AI Platform!** Experience the power of artificial intelligence ...</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>2026-07-02T18:43:33Z</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=vAxlkLjP-Xs</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Welcome to SmartAISchool! 🚀</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Dive into the world of Artificial Intelligence, tech trends, and digital skills with us! From AI tutorials, tool reviews, and industry ...</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>2026-07-06T04:50:00Z</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=GRPzhZPzV0g</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>My firmware for livestream projects with AI features.</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Hello everyone! This test-mode livestream is launched to verify stable workflow of my own software for live streaming in a high ...</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>2026-04-20T21:23:11Z</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=_dyOinvkmIc</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>XAUUSD LIVE AI FOREX TRADING 06-07-2026 -- FRANK H1 BOT #forex #frankbot #xauusd #bot</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Frank Bot – Live Automated Forex Trading Frank Bot is a fully automated Forex trading system built to execute a proven ...</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2026-07-06T10:16:46Z</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=VB6VTeI3Hek</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>🔴LIVE: Fable 5 vs Gemini 3.1 AI Trading EA on XAUUSD (MT5/MT4) — DoIt Alpha Pulse AI</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>LIVE forward test of my AI Trading EA for MetaTrader 5 / MetaTrader 4: DoIt Alpha Pulse AI. Today we're also testing Gemini 3.1 ...</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>2026-06-26T08:13:18Z</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=DFnrNNTJ4Vk</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Make Money With Claude AI — The Complete FREE Course (24/7 Live)</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>The complete FREE course on making money with Claude AI — now running 24/7. 16 modules, 90 minutes, on loop. ▷ Watch the ...</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>2026-07-04T10:16:43Z</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=tkMFq7Jrr2Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Live News &amp;amp; World Events — 24/7 | Defaxon Live (English)</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Defaxon Live — 24/7 AI World-Event Intelligence A live, AI-curated map of what's happening on Earth — every domain, every ...</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>2026-06-27T09:16:18Z</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=E20okCc9MOQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>🔴 LIVE: 100+ AI Agents Trading ETH Futures | Real PNL 24/7</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Trading Wars — Clash of Agents 100+ autonomous AI agents battle every 5 minutes to win the next trade. Watch AI agents ...</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>2026-06-16T18:07:58Z</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=PcWuca4Q6Dc</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>AI Automation Masterclass - Demo for Small Businesses &amp; ...</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>AI Automation Masterclass - Demo for Small Businesses &amp; ...
+Eventbrite
+https://www.eventbrite.com › ai-auto...</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Webinar: AI Automation Processes – How to Boost Efficiency ...</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Webinar: AI Automation Processes – How to Boost Efficiency ...
+YouTube · HYVE
+&gt;60 lượt xem: · 8 tháng trước</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>AI Automation Fundamentals: An Introduction to Zapier &amp; ...</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>AI Automation Fundamentals: An Introduction to Zapier &amp; ...
+Eventbrite
+https://www.eventbrite.com › ai-auto...</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>FHMoms Free Webinar AI Automation Webinar with live demo ...</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>FHMoms Free Webinar AI Automation Webinar with live demo ...
+YouTube · Filipina Homebased Moms
+&gt;530 lượt xem: · 4 tháng trước</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>AI Automation Masterclass Replay, n8n Training &amp; AI ...</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>AI Automation Masterclass Replay, n8n Training &amp; AI ...
+YouTube · Solomon Christ AI + Automation Mastery
+&gt;740 lượt xem: · 1 tháng trước</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>AI Automation Full Course 2026 [FREE] | AI Automation ...</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>AI Automation Full Course 2026 [FREE] | AI Automation ...
+YouTube · Simplilearn
+&gt;31,8 N lượt xem: · 1 tháng trước</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Be WOWED by Live AI &amp; Automation — Watch It Build and ...</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Be WOWED by Live AI &amp; Automation — Watch It Build and ...
+Eventbrite
+https://www.eventbrite.com › be-wow...</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>AI + Automation Study Hall Live, n8n Workflows &amp; Business AI</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>AI + Automation Study Hall Live, n8n Workflows &amp; Business AI
+YouTube · Solomon Christ AI + Automation Mastery
+&gt;120 lượt xem: · 2 ngày trước</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>AI Systems with Crew AI: Build Powerful Automation | Live ...</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>AI Systems with Crew AI: Build Powerful Automation | Live ...
+YouTube · Interview Kickstart India
+&gt;100 lượt xem: · 3 tuần trước</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: filter out stale events (UPCOMING 4 years ago bug) - add time_filter_events, fix YouTube is_valid_event, fix Meetup date filtering
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3093,12 +3093,420 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>[Tutorial] Create a Charity Livestream Event Using Twitch and ...</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>[Tutorial] Create a Charity Livestream Event Using Twitch and ...
+YouTube · Point of Pride
+&gt;240 lượt xem: · 4 năm trước</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>{LIVESTREAM} Charity Livestream! #ColouringForCancer ...</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>{LIVESTREAM} Charity Livestream! #ColouringForCancer ...
+YouTube · Axik Fumbles
+&gt;1,1 N lượt xem: · 5 tháng trước</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Charity Livestream 2023</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Charity Livestream 2023
+YouTube
+https://m.youtube.com › playlist</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Charity Livestream TerraFirmaCraft Part 1 of 2</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Charity Livestream TerraFirmaCraft Part 1 of 2
+Twitch · kijkers
+&gt;1,6 N lượt xem: · 13 năm trước</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>OpenFront Charity Livestream!</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>OpenFront Charity Livestream!
+YouTube · Ultimus_Rex
+&gt;7,4 N lượt xem: · 6 tháng trước</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Charity livestream(noch zu sortieren)</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Charity livestream(noch zu sortieren)
+YouTube Music
+https://music.youtube.com › playlist</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>E Sports Charity Livestream</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>E Sports Charity Livestream
+YouTube · Suffolk New College
+&gt;10 lượt xem: · 2 tháng trước</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>How To Run A Successful Charity Livestream - 7 Tips</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>How To Run A Successful Charity Livestream - 7 Tips
+YouTube · Gaming Careers
+&gt;28,4 N lượt xem: · 7 năm trước</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Fallout 4 Hope | Charity LIVE Stream</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Fallout 4 Hope | Charity LIVE Stream
+YouTube · Gopher
+&gt;3,2 N lượt xem: · 1 tuần trước</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Extra Life Charity Live Stream 2024</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Extra Life Charity Live Stream 2024
+YouTube · Aaron Longstaff
+&gt;3,2 N lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Finding Pride! A Charity Live Stream Event June 14th! Time TBA!</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Finding Pride! A Charity Live Stream Event June 14th! Time TBA!
+YouTube · BogWitchSophie
+3 lượt xem · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Fallout 4 Hope | Charity LIVE Stream !donate</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Fallout 4 Hope | Charity LIVE Stream !donate
+YouTube · Gopher
+&gt;4,3 N lượt xem: · 5 ngày trước</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>First Charity Live Stream Event - Hilarious Highlights</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>First Charity Live Stream Event - Hilarious Highlights
+YouTube · LPX Tech
+&gt;140 lượt xem: · 11 năm trước</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>charitylivestream</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>charitylivestream
+YouTube
+https://www.youtube.com › hashtag › c...</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Alex Hirsch &amp; Pals BIG CHARITY DRAW-A-THON for the LA ...</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Alex Hirsch &amp; Pals BIG CHARITY DRAW-A-THON for the LA ...
+YouTube · TheMysteryofGF
+&gt;188,4 N lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Whitney Teaches Sam Burlesque | Sam's 24-Hour Charity ...</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Whitney Teaches Sam Burlesque | Sam's 24-Hour Charity ...
+YouTube · Critical Role
+&gt;45,4 N lượt xem: · 2 tháng trước</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Sharing is Caring | Charity #live #livestream #philippines ...</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Sharing is Caring | Charity #live #livestream #philippines ...
+YouTube · FARMGIRL NG ISABELA
+&gt;1,5 N lượt xem: · 2 tuần trước</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: show results across topic changes - remove DB dedup from search results, fix YouTube is_valid_event to not reject events without timestamp
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J123"/>
+  <dimension ref="A1:J129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3501,12 +3501,156 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Charity Network Webinar: Building Your Voice &amp; Visibility</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Charity Network Webinar: Building Your Voice &amp; Visibility
+eventbrite.com
+https://www.eventbrite.com › charity-...</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Webinar: Is your charity AI ready? [Hear from a real range ...</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Webinar: Is your charity AI ready? [Hear from a real range ...
+Eventbrite
+https://www.eventbrite.com › webinar...</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Best Charity &amp; Causes Seminar Online - Events &amp; Activities</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Best Charity &amp; Causes Seminar Online - Events &amp; Activities
+Eventbrite
+https://www.eventbrite.com › online › charity-and-caus...</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Charity &amp; Causes events Online</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Charity &amp; Causes events Online
+Eventbrite
+https://www.eventbrite.com › Online › Online Events</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>YPI Charity Webinar September 2024</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>YPI Charity Webinar September 2024
+Vimeo
+https://vimeo.com › ... › Videos</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Charity Webinar - Fundraising Events 2025</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Charity Webinar - Fundraising Events 2025
+YouTube · Eventmaster
+&gt;50 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: filter stale UPCOMING events by year in title/description (2024, 2025 events showing as UPCOMING)
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J129"/>
+  <dimension ref="A1:J147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3645,12 +3645,444 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Small Charity Week 2026: Fundamentals of Fundraising webinar</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Small Charity Week 2026: Fundamentals of Fundraising webinar
+YouTube · Big Give
+&gt;70 lượt xem: · 1 tháng trước</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Plan a Perfect Charity Event in 14 Steps</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Plan a Perfect Charity Event in 14 Steps
+Eventbrite
+https://www.eventbrite.com › blog › h...</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Small Charity Week 2025: Application Webinar</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Small Charity Week 2025: Application Webinar
+YouTube · Big Give
+&gt;920 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Twitch's Charity Tool for Creators</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Twitch's Charity Tool for Creators
+Twitch
+https://help.twitch.tv › twitch-charity</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>How to Organise a Charity Fundraising Event (UK Fundraising ...</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>How to Organise a Charity Fundraising Event (UK Fundraising ...
+YouTube · Evolve Catalyst | Charity Management Consultancy
+&gt;200 lượt xem: · 4 tháng trước</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>OVER 2,000 PEOPLE PARTICIPATE IN CHARITY WALK AND ...</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>OVER 2,000 PEOPLE PARTICIPATE IN CHARITY WALK AND ...
+YouTube · HTV Tin Tức
+&gt;280 lượt xem: · 1 tuần trước</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>How to Run a Successful Charity Livestream</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>How to Run a Successful Charity Livestream
+YouTube · Funds2Orgs
+&gt;370 lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Mastering Charity Events: Your Ultimate Guide to Making a ...</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Mastering Charity Events: Your Ultimate Guide to Making a ...
+YouTube · Event Crowd
+&gt;120 lượt xem: · 2 năm trước</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>How to Set Clear Goals for a Successful Charity Event</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>How to Set Clear Goals for a Successful Charity Event
+YouTube
+https://m.youtube.com › shorts</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Panel Discussion - The evolution of event fundraising</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Panel Discussion - The evolution of event fundraising
+YouTube · Charity Digital
+&gt;20 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>What is Livestream Fundraising? | Funraise Nonprofit ...</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>What is Livestream Fundraising? | Funraise Nonprofit ...
+YouTube · Funraise
+&gt;240 lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Fundraising Ideas for Live Streaming Online</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Fundraising Ideas for Live Streaming Online
+YouTube · PTZOptics
+&gt;350 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>How To Use Facebook Live For Fundraising Events</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>How To Use Facebook Live For Fundraising Events
+YouTube · Aplos
+&gt;1,5 N lượt xem: · 5 năm trước</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>How to do a virtual livestream fundraiser with Eventgroove ...</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>How to do a virtual livestream fundraiser with Eventgroove ...
+YouTube · Eventgroove
+&gt;160 lượt xem: · 4 năm trước</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>The New Telethon How Live Streaming Has Changed ...</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>The New Telethon How Live Streaming Has Changed ...
+YouTube · Neon One
+&gt;360 lượt xem: · 5 năm trước</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Livestream Fundraising — With Max (CEO) &amp; Tori (Customer ...</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Livestream Fundraising — With Max (CEO) &amp; Tori (Customer ...
+YouTube · Givebutter
+&gt;1,8 N lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Facebook Live Fundraising Best Practices for Nonprofits ...</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Facebook Live Fundraising Best Practices for Nonprofits ...
+YouTube · MobileCause now GiveSmart
+&gt;2 N lượt xem: · 9 năm trước</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>How to Increase Attendance at Your Next Fundraising Event ...</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>How to Increase Attendance at Your Next Fundraising Event ...
+YouTube · MobileCause now GiveSmart
+&gt;9,6 N lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: improve year-in-title filter to scan all statuses without timestamps
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J147"/>
+  <dimension ref="A1:J165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4077,12 +4077,444 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
-      <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>[webinar] Online Event Fundraiser: Lessons to Share</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>[webinar] Online Event Fundraiser: Lessons to Share
+Vimeo
+https://vimeo.com › ... › Videos</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>[Webinar] Hit your fundraising goals without hosting another ...</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>[Webinar] Hit your fundraising goals without hosting another ...
+YouTube · Givebutter
+&gt;330 lượt xem: · 3 tháng trước</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Monthly trending searches in 67199, Australia Newport</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Monthly trending searches in 67199, Australia Newport
+Eventbrite
+https://www.eventbrite.com › trending › australia--new...</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Charity Fundraiser LIVESTREAM for Mental Health w ...</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Charity Fundraiser LIVESTREAM for Mental Health w ...
+YouTube · Stuff &amp; Whiskey
+&gt;3,1 N lượt xem: · 3 năm trước</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>EPIC Fundraiser Stream for Children's Healthcare</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>EPIC Fundraiser Stream for Children's Healthcare
+YouTube · Jorge Rivera-Herrans
+&gt;167,3 N lượt xem: · 4 tháng trước</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Pledge.to Guide: How to Create a Live Event Display</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Pledge.to Guide: How to Create a Live Event Display
+YouTube · Pledge
+&gt;190 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Stream #WithMe Live Event | Creator Fundraiser</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Stream #WithMe Live Event | Creator Fundraiser
+YouTube · YouTube Originals
+6 năm trước</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>(PAST LIVESTREAM) #TeamSeas Live Count ($30 Million ...</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>(PAST LIVESTREAM) #TeamSeas Live Count ($30 Million ...
+YouTube · YT Battles
+4 năm trước</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>How to Start a Charity Live Stream | Streamlabs</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>How to Start a Charity Live Stream | Streamlabs
+YouTube · Streamlabs
+&gt;17,6 N lượt xem: · 5 năm trước</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Lands Between Fundraiser Stream Benefiting KOI</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Lands Between Fundraiser Stream Benefiting KOI
+YouTube · Noah Caldwell-Gervais
+&gt;10 N lượt xem: · 3 tuần trước</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Massive Holiday Livestream 2025!</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Massive Holiday Livestream 2025!
+YouTube · 3D Printing Nerd
+&gt;26,9 N lượt xem: · 6 tháng trước</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>EPIC Fundraiser Stream for Children's Healthcare Pt. 2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>EPIC Fundraiser Stream for Children's Healthcare Pt. 2
+YouTube · Jorge Rivera-Herrans
+&gt;93,1 N lượt xem: · 4 tháng trước</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>*• TRUTH or DARE – PRIDE LIVESTREAM FUNDRAISER ...</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>*• TRUTH or DARE – PRIDE LIVESTREAM FUNDRAISER ...
+YouTube · Not-So-Average-Fangirl
+&gt;21,8 N lượt xem: · 1 tuần trước</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>One song, millions raised: The phenomenon of the Polish ...</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>One song, millions raised: The phenomenon of the Polish ...
+YouTube · TVP WORLD
+&gt;10,3 N lượt xem: · 2 tháng trước</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>24 Hour Livestream Fundraiser Event Announcement for CMN ...</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>24 Hour Livestream Fundraiser Event Announcement for CMN ...
+YouTube · DarkTaker1990
+&gt;20 lượt xem: · 4 tuần trước</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>T-Ball Under the Lights Livestream Fundraiser</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>T-Ball Under the Lights Livestream Fundraiser
+YouTube · HPS Stream Team
+4 ngày trước</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>PET NEEDS Van Fundraiser Livestream</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>PET NEEDS Van Fundraiser Livestream
+YouTube · PET NEEDS
+&gt;560 lượt xem: · 10 tháng trước</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>One Beating Heart: A Livestream Fundraiser for Covid-19 ...</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>One Beating Heart: A Livestream Fundraiser for Covid-19 ...
+YouTube · The Midnight
+&gt;70,5 N lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr"/>
+      <c r="J165" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: raise relevance threshold to 10, tighten platform trust boost to require title keyword match
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J165"/>
+  <dimension ref="A1:J235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4509,12 +4509,1451 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
-      <c r="H165" t="inlineStr"/>
-      <c r="I165" t="inlineStr"/>
-      <c r="J165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Tokenization Webinar with Apex Capital</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Tokenization Webinar with Apex Capital
+Eventbrite
+https://www.eventbrite.com › tokeniza...</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Webinar: Tokenization in the UAE</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Webinar: Tokenization in the UAE
+YouTube · DigiShares
+&gt;480 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Real-World Asset Tokenization | 2-Hour Online Workshop</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Real-World Asset Tokenization | 2-Hour Online Workshop
+Eventbrite
+https://www.eventbrite.com › real-wor...</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Unlocking the Future: Tokenization Webinar with Innowise's ...</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Unlocking the Future: Tokenization Webinar with Innowise's ...
+YouTube · Innowise Global
+&gt;380 lượt xem: · 2 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Real Estate Tokenization Webinar with Aurora Cloud</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Real Estate Tokenization Webinar with Aurora Cloud
+YouTube · Aurora
+&gt;440 lượt xem: · 2 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Tokenization Webinar with Alex Chan</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Tokenization Webinar with Alex Chan
+YouTube
+https://www.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Learning with LEVERAGE: Tokenization Webinar, January 10 ...</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Learning with LEVERAGE: Tokenization Webinar, January 10 ...
+YouTube · LeagueofSECUs
+&gt;80 lượt xem: · 3 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>EMV Tokenization Webinar</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>EMV Tokenization Webinar
+YouTube · Secure Technology Alliance
+&gt;17,2 N lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Financial security tokenization, Fri, Jul 3, 2026, 12:00 AM</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Financial security tokenization, Fri, Jul 3, 2026, 12:00 AM
+Meetup
+https://www.meetup.com › events</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>EN | Real World Asset Tokenization Live Use Cases Across ...</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>EN | Real World Asset Tokenization Live Use Cases Across ...
+YouTube · MERGE
+&gt;20 lượt xem: · 2 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>XRP CRYPTO TOKENIZATION LIVE NOW!!!!!</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>XRP CRYPTO TOKENIZATION LIVE NOW!!!!!
+YouTube · Oscar Ramos
+&gt;15,2 N lượt xem: · 3 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Explore Tokenization with the DigiShares Webinar Series</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Explore Tokenization with the DigiShares Webinar Series
+YouTube · DigiShares
+&gt;60 lượt xem: · 2 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>How to Tell If Your Asset Is Ready for Tokenization — Live ...</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>How to Tell If Your Asset Is Ready for Tokenization — Live ...
+YouTube · Stobox
+&gt;130 lượt xem: · 1 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Adversarial Tokenization</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Adversarial Tokenization
+YouTube
+&gt;40 lượt xem: · 11 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>GeneticBPE: Motif-Preserving Tokenization for Robust miRNA ...</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>GeneticBPE: Motif-Preserving Tokenization for Robust miRNA ...
+YouTube
+&gt;20 lượt xem: · 11 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Webinars</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Webinars
+YouTube · DigiShares
+&gt;2,1 N người theo dõi</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Beyond the Hype:Top 3 Risk-First Applications of ...</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Beyond the Hype:Top 3 Risk-First Applications of ...
+Eventbrite
+https://www.eventbrite.com › beyond-...</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Token Cost Management: Bringing Spend Under Control</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Kong/HO-CHI-MINH-CITY
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Tue, Jul 21 · 10:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/kong-ho-chi-minh-city/events/315576574/</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>&lt;Free Online Event&gt;International exchange (Only Japanese language)✨日本語だけで国際交流</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Enjoy Japanese!  Vietnam　～日本語だけの国際交流会～
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Every Wed · Jul 8 · 7:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/online-enjoy-nihongo-vietnam-other-14-countries/events/315312113/</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Global - Dev Automation and Harness Engineering I</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Advanced AI Concepts-Ho Chi Minh City
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Sun, Jul 12 · 9:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/advanced-ai-concepts-ho-chi-minh-city/events/315556791/</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Global - Anthropic Certified Architect Prep</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Advanced AI Concepts-Ho Chi Minh City
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Sun, Jul 19 · 9:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/advanced-ai-concepts-ho-chi-minh-city/events/315538127/</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Anthropic Certified Architect Prep</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Advanced AI Concepts-Ho Chi Minh City
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Sat, Jul 18 · 7:00 AM ICT</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/advanced-ai-concepts-ho-chi-minh-city/events/315536180/</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Get Leads Online with AI (Live Workshop Preview)</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Internet Entrepreneurs Network (Vietnam)
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Thu, Jul 9 · 10:00 AM ICT</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/internet-entrepreneurs-network-vietnam/events/315497013/</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Saigon Sunday Free Online Guided Meditation- Beginners and Intermediate</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Organizer: Saigon Sahaja Yoga Meditation
+Attendees: 4 attendees</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Every Sun · Jul 12 · 8:45 AM ICT</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/saigon-meditation/events/315566317/</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Khoá Học Professional Scrum Master (PSM) - Lớp Online</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Scrum Day Vietnam
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Sat, Jul 25 · 9:00 AM ICT</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/scrum-day-vietnam/events/315264764/</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Beginners Free Online Guided Meditation and Follow-Up</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Organizer: Saigon Sahaja Yoga Meditation
+Attendees: 5 attendees</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Every Sun · Jul 12 · 8:45 PM ICT</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/saigon-meditation/events/315368406/</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>AI Governance for AI Developers</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Advanced AI Concepts-Ho Chi Minh City
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Sat, Jul 25 · 7:00 AM ICT</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/advanced-ai-concepts-ho-chi-minh-city/events/315538437/</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Global - AI Governance for AI Developers</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Advanced AI Concepts-Ho Chi Minh City
+Attendees: </t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Sun, Jul 26 · 9:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/advanced-ai-concepts-ho-chi-minh-city/events/315538596/</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>African Roof Top Solar Makes Families Money #EDMA #bitcoin ...</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>African Roof Top Solar Makes Families Money #EDMA #bitcoin ...
+YouTube
+https://www.youtube.com › shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>LIVE from Dubai: Why RWAs Are Dominating Token2049 + ...</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>LIVE from Dubai: Why RWAs Are Dominating Token2049 + ...
+YouTube · Action Crypto
+&gt;1,2 N lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Webinar with CEO of DigiU: RWA-Marketplace</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Webinar with CEO of DigiU: RWA-Marketplace
+YouTube · DIGIU
+&gt;16 N người theo dõi</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>RWA Day NYC</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>RWA Day NYC
+lu.ma
+https://lu.ma › rwa</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Tokenized RWA Bootcamp</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Tokenized RWA Bootcamp
+lu.ma
+https://lu.ma › Tokenized-RWA-bootc...</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Bridging the Trillion: Institutional RWA Tokenization Meets ...</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Bridging the Trillion: Institutional RWA Tokenization Meets ...
+Eventbrite
+https://www.eventbrite.com › bridgin...</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>RWA</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>RWA
+Vimeo
+https://vimeo.com › user212606547</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>RWA Live @ Korea Buidl Week</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>RWA Live @ Korea Buidl Week
+lu.ma
+https://lu.ma › ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>20/20 in Maths| RWA Live Mock 28 June 26 Complete ...</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>20/20 in Maths| RWA Live Mock 28 June 26 Complete ...
+YouTube · Learn with HiM
+&gt;1,2 N lượt xem: · 1 tuần trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>RWA Live Mock 05 July 2026 Maths Solution | Score 20/20 ...</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>RWA Live Mock 05 July 2026 Maths Solution | Score 20/20 ...
+YouTube · Learn with HiM
+&gt;250 lượt xem: · 1 ngày trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 1</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 1
+YouTube
+https://m.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 3</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 3
+YouTube
+https://m.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>SSC GD 2026 | RWA Live Mock 25 January 2026 maths ...</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>SSC GD 2026 | RWA Live Mock 25 January 2026 maths ...
+YouTube · math with praveen bajpai
+&gt;900 lượt xem: · 5 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>RWA Live 4 Main Event Cipriano Abruzzi vs T Phoenix pt 1</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>RWA Live 4 Main Event Cipriano Abruzzi vs T Phoenix pt 1
+YouTube · Renegade Wrestling Alliance
+&gt;140 lượt xem: · 15 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>RWA Live ´03 Video VEGAS 4 FREE</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>RWA Live ´03 Video VEGAS 4 FREE
+YouTube · Rings of Europe - PRO Wrestling
+&gt;710 lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>RWA Livestream with Townsquare &amp; Monad</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>RWA Livestream with Townsquare &amp; Monad
+YouTube
+https://www.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>$TX Talk 🎙️ Late Night tx Market and RWA Livestream</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>$TX Talk 🎙️ Late Night tx Market and RWA Livestream
+YouTube
+https://www.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>AURUM NEO BANK and GOLD RWA (Webinar 16 April 2026)</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>AURUM NEO BANK and GOLD RWA (Webinar 16 April 2026)
+YouTube
+https://www.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Biology Vs Chemistry ⚗️ | Life Vs Lab Showdown | RWA ...</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Biology Vs Chemistry ⚗️ | Life Vs Lab Showdown | RWA ...
+YouTube · UP Board English Medium RWA
+&gt;3,4 N lượt xem: · 11 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>naveen sir fan #naveen #rwa #livestream #rwaclasses #aakitsir ...</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>naveen sir fan #naveen #rwa #livestream #rwaclasses #aakitsir ...
+YouTube
+https://www.youtube.com › shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Renegade Wrestling Alliance</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Renegade Wrestling Alliance
+YouTube · Renegade Wrestling Alliance
+&gt;2,8 N người theo dõi</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Free Career Empowerment &amp; Meditation Class</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Organizer: Free Career Empowerment &amp; Meditation Series
+Attendees: 2 attendees</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Every Wed · Jul 8 · 7:30 AM ICT</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/hanoi-career-empowerment-meditation-series/events/315509530/</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Bridging the Trillion: Institutional RWA Tokenization Meets ...</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Bridging the Trillion: Institutional RWA Tokenization Meets ...
+Eventbrite
+https://www.eventbrite.com › bridgin...</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>[Webinar] Growing Tezos Ecosystem with RWA Tokenization &amp; ...</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>[Webinar] Growing Tezos Ecosystem with RWA Tokenization &amp; ...
+YouTube
+https://m.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Webinar: RWA Tokenization on Provenance, Polygon, Liquid ...</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Webinar: RWA Tokenization on Provenance, Polygon, Liquid ...
+YouTube · DigiShares
+&gt;380 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>RWA Tokenization: Why 2026 Matters</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>RWA Tokenization: Why 2026 Matters
+YouTube · Brickken
+&gt;70 lượt xem: · 4 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>RWA Live @ Korea Buidl Week</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>RWA Live @ Korea Buidl Week
+lu.ma
+https://lu.ma › ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>20/20 in Maths| RWA Live Mock 28 June 26 Complete ...</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>20/20 in Maths| RWA Live Mock 28 June 26 Complete ...
+YouTube · Learn with HiM
+&gt;1,2 N lượt xem: · 1 tuần trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>RWA Live Mock 05 July 2026 Maths Solution | Score 20/20 ...</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>RWA Live Mock 05 July 2026 Maths Solution | Score 20/20 ...
+YouTube · Learn with HiM
+&gt;250 lượt xem: · 1 ngày trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 1</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 1
+YouTube
+https://m.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 3</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>RWA Live 5 Main Event The Agency vs The Abruzzis pt 3
+YouTube
+https://m.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>SSC GD 2026 | RWA Live Mock 25 January 2026 maths ...</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>SSC GD 2026 | RWA Live Mock 25 January 2026 maths ...
+YouTube · math with praveen bajpai
+&gt;900 lượt xem: · 5 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>RWA Live 4 Main Event Cipriano Abruzzi vs T Phoenix pt 1</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>RWA Live 4 Main Event Cipriano Abruzzi vs T Phoenix pt 1
+YouTube · Renegade Wrestling Alliance
+&gt;140 lượt xem: · 15 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>RWA Live ´03 Video VEGAS 4 FREE</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>RWA Live ´03 Video VEGAS 4 FREE
+YouTube · Rings of Europe - PRO Wrestling
+&gt;710 lượt xem: · 6 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>RWA Livestream with Townsquare &amp; Monad</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>RWA Livestream with Townsquare &amp; Monad
+YouTube
+https://www.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>$TX Talk 🎙️ Late Night tx Market and RWA Livestream</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>$TX Talk 🎙️ Late Night tx Market and RWA Livestream
+YouTube
+https://www.youtube.com › watch</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Tokenization in the U.S. Webinar | Expert Panel Discussion</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Tokenization in the U.S. Webinar | Expert Panel Discussion
+YouTube · DigiShares
+&gt;510 lượt xem: · 6 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Tokenizing commodities &amp; RWAs presented by zenGate Global</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Tokenizing commodities &amp; RWAs presented by zenGate Global
+YouTube · Cardano Foundation
+&gt;960 lượt xem: · 2 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Biology Vs Chemistry ⚗️ | Life Vs Lab Showdown | RWA ...</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Biology Vs Chemistry ⚗️ | Life Vs Lab Showdown | RWA ...
+YouTube · UP Board English Medium RWA
+&gt;3,4 N lượt xem: · 11 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>naveen sir fan #naveen #rwa #livestream #rwaclasses #aakitsir ...</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>naveen sir fan #naveen #rwa #livestream #rwaclasses #aakitsir ...
+YouTube
+https://www.youtube.com › shorts</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Webinars</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Webinars
+YouTube · DigiShares
+&gt;2,1 N người theo dõi</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Renegade Wrestling Alliance</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Renegade Wrestling Alliance
+YouTube · Renegade Wrestling Alliance
+&gt;2,8 N người theo dõi</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr"/>
+      <c r="H235" t="inlineStr"/>
+      <c r="I235" t="inlineStr"/>
+      <c r="J235" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
optimize event collection with streaming, memoization, and persistent filtering
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livestreams" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Livestreams" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J235"/>
+  <dimension ref="A1:J236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5947,13 +5947,30 @@
 &gt;2,8 N người theo dõi</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
-      <c r="G235" t="inlineStr"/>
-      <c r="H235" t="inlineStr"/>
-      <c r="I235" t="inlineStr"/>
-      <c r="J235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Test Event</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr"/>
+      <c r="D236" t="inlineStr"/>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=unique123</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr"/>
+      <c r="H236" t="inlineStr"/>
+      <c r="I236" t="inlineStr"/>
+      <c r="J236" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add active spam learning and session-persisted UI
Introduce two new AI scoring modules: an active-learning spam classifier trained from user feedback, and a cross-encoder relevance scorer for goal-to-event semantic matching. Wire both into `services/relevance_filter.py` so spam can be filtered early and semantic confidence can boost relevance scoring.

Update `dashboard/streamlit_app.py` to persist search results in `st.session_state` across reruns, render saved results consistently, and add per-event feedback controls (thumbs up/down) that write training data and optionally remove spam-marked items from the current result list.
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O29"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1788,12 +1788,1387 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
-      <c r="O29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>[webinar] Online Event Fundraiser: Lessons to Share</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>48</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Fundarise Livestream</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>For organizations with limited online presence, what strategies have you found most effective in leveraging social media to promote online events and drive ticket sales?</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>[webinar] Online Event Fundraiser: Lessons to Share
+Vimeo
+https://vimeo.com › ... › Videos</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Best 1 RWA tokenization platforms - S-PRO</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>55</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Tokenization</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người?</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Best 1 RWA tokenization platforms - S-PROS-PROhttps://s-pro.io › rwa-tokenization-platforms</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Tokenization Protocols - Meegle</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>55</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Tokenization</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Have you considered the implications of tokenization on data governance, particularly in regulated industries like finance where data residency and sovereignty are major concerns?</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Tokenization Protocols - MeegleMeeglehttps://www.meegle.com › en_us › topics › tokenization-...</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>[Webinar] Hit your fundraising goals without hosting another ...</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>71</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Organization Manager</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Charity</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người?</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>[Webinar] Hit your fundraising goals without hosting another ...
+YouTube · Givebutter
+&gt;330 lượt xem: · 3 tháng trước</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Fund Tokenization: Building Bridges in Global Fund Distribution</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>55</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Tokenization</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>How do you see tokenization addressing the issue of fragmented fund ownership structures, which can lead to inefficient distribution and high costs for investors?</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Fund Tokenization: Building Bridges in Global Fund Distribution
+Nicsa
+https://nicsa.org › product › fund-tok...</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>🔴 LIVE | Fundraiser for Jantar Mantar Students | Every Donation Makes a Difference ❤️</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>165</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Gamers and philanthropists</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>How will the funds raised from this BGMI charity stream be allocated to support the students at Jantar Mantar, are there any specific programs or initiatives that will be prioritized? | I'd love to know more about the current challenges faced by the students at Jantar Mantar and how this charity stream aims to address them, are there any specific stories or examples you can share? | Will there be any opportunities for donors to get involved beyond just contributing financially, such as volunteering or mentoring the students at Jantar Mantar?</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>LIVE BGMI Charity Stream | Supporting Students at Jantar Mantar ❤️     Welcome to today's **BGMI LIVE Charity Stream!</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:33:34Z</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=djx068LuF4Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>LIVE Fundraiser Minecraft and Heal behind the scenes in real life of a nonprofit</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>145</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Philanthropist/Gamer</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Nonprofit</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>I'm curious to know how the Eudaimonia Project Film Festival plans to allocate the donated funds, will they be used for specific programs or general operational costs? | How does the nonprofit plan to measure the impact of the fundraiser, are there any specific metrics or outcomes they're hoping to achieve with the donations? | Are there any plans to collaborate with other nonprofits or organizations in the charity sector to amplify the effects of the fundraiser and the film festival?</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Please Donte https://live.givebutter.com/c/the-eudaimonia-project-film-festival-b2vu4h.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:33:44Z</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=OTqbl8UnInE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>🔴 LIVE CHARITY STREAM | Save Little Krishna ❤️ Every Donation Can Save a Life 🙏</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>145</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Empathetic Donor</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Non-Profit/Healthcare</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>What's the current status of Little Krishna's treatment and how will the donations from this stream be allocated to support his medical expenses? | Are there any plans for long-term support or follow-up care for Little Krishna after the initial treatment, and how can we as a community continue to help? | Can you share more about the specific medical condition Little Krishna is facing and what the prognosis is with timely and proper treatment, so we can better understand the urgency of the situation?</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Please Help Save Little Krishna Little Krishna is fighting a serious medical condition and urgently needs support for treatment.</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2026-07-21T15:35:00Z</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=I0yjeB8Tqf4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>the andrew nocturnna and wEndy charity stream</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>110</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>supporter/donor</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>gaming/charity</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Just donated to the GoFundMe campaign, hoping Andrew gets the support he needs - what's the current status on his housing situation? | How will the funds raised from this stream be allocated to support Andrew's rehabilitation and education? | Are there any plans for long-term support or mentorship programs for Andrew and others who've experienced similar situations, perhaps through partnerships with local charities?</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>the gofundme fundraiser: https://www.gofundme.com/f/andrew-hospitalized-by-abusive-parents-now-homeless.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>2026-01-13T05:40:03Z</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=tETQ11QlHGo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>pls donate</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>83</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Charity</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>What's the primary cause that this charity is supporting, and how will the donated funds be allocated? | Are there any specific donation milestones or targets that we can help reach during this livestream? | Will there be any matching donations or sponsorships to amplify the impact of our contributions?</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:00:19Z</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=P3-fKqN2b8A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Wolf&amp;#39;s Den Takeover Tuesday of the AGB Charity channel on kick!! !AGB !face !AGB !face</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>80</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Gamers, particularly those interested in charity events and community engagement</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Love the gaming for a cause concept, how does the AGB Charity channel plan to allocate donations from tonight's stream? | MnK, what's your strategy for tackling tough levels in the games you're playing, and will you be taking donations for specific charity milestones? | Will the stream be featuring any charity-specific games or challenges, like a 'donate to skip' level or a 'charity boss fight'?</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>MnK old Fart playing some Games.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:52:24Z</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=uMuJEqYyFr0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>deep focus lofi radio 🎯 24/7 charity beats for deep work (live now)</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>80</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Students, programmers, and individuals seeking focus or relaxation</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Music/Entertainment</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>I've noticed the lofi beats have a calming effect, do you think the same tracks could be used in therapy sessions for anxiety relief in homeless shelters? | How does the donation process work - is it a fixed amount per listener or based on the total hours streamed? | Are there any plans to collaborate with mental health professionals to create customized lofi playlists for specific conditions, like PTSD, which is common among the homeless population?</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>24/7 Lofi beats for deep focus, sleep, and anxiety relief. Every minute you listen helps provide real support for the homeless.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>2026-07-21T10:00:07Z</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=5vgTpAWTqy4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>🔴CHARITY🔴DONATE = CHANGE THE GAME🔴GEOMETRY DASH TRIATHLON</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>80</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Gamers, charity supporters</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>How does the donation tier system work in terms of unlocking exclusive rewards in the Geometry Dash triathlon? | I'm curious to know if there are any specific charity initiatives or causes that the Globed Room 360648 is supporting through this event? | Are there any plans to offer additional challenges or bonus levels for donors who contribute above a certain amount, similar to the ones mentioned in the Challenge Info section?</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Donate here: https://charity.gd/gdce/ Globed Room: 360648 Challenge Info   Depending on the amount donated, you can buy ...</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=woFm1lBy8cE</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>God says&amp;quot; Today Marks the End of That Affliction | Evang Charity Odochi is live!</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>80</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Individuals seeking spiritual guidance or solace</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Religion/Spirituality</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Evang Charity, what role do you believe faith-based organizations can play in addressing systemic afflictions, such as poverty and inequality, in our communities? | Can you share an example of a successful charity initiative that you've been involved with, and how it's helped alleviate affliction for a specific group of people? | How do you think we can balance spiritual guidance with tangible support in charity work, to ensure we're making a lasting impact on those we're trying to help?</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>God says" Today Marks the End of That Affliction | Evang Charity Odochi is live!</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>2026-07-21T13:35:36Z</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=wVHnJwaSpWI</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ready For Battle⚔️🛡️ || Kidz Family Camp 2026 || Pastor Charity Kalstrup</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>80</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Christian families with children</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Pastor Charity, how do you think the Kidz Family Camp 2026 can be used as a platform to raise awareness and funds for local charities, particularly those supporting underprivileged kids? | I'm curious to know more about the chooselife Kidz Ministry's outreach programs - are there any plans to collaborate with other organizations to amplify the impact of the Kidz Family Camp? | What role do you envision the church community playing in supporting the Kidz Family Camp, and are there opportunities for volunteers to get involved in the planning and execution process?</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>This message was recorded live at chooselife CHURCH in Hobbs, NM. For more information about Chooselife Kidz Ministry visit ...</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2026-07-21T16:00:00Z</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=pQS1z_hYIco</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Charity Cup Mini S-10</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>80</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Gamers, Esports enthusiasts</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>How does the Charity Cup Mini S-10 format impact donor engagement, particularly in terms of repeat participation? | What's the strategy behind using #PRISMLiveStudio for this event, and how does it enhance the overall charity experience? | Are there any plans to offer virtual participation options for the Charity Cup Mini S-10, to expand the reach and inclusivity of the event?</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>This stream is created with #PRISMLiveStudio.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>2026-07-21T16:18:41Z</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Mod7A6OTwZw</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Breaking News LIVE | Current Affairs News | CJP Protest | Headlines | Ram Mandir Donation</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>75</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Individuals interested in current events and news, particularly those from India or with an interest in Indian affairs</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>News/Media</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Curious to know how the Ram Mandir donation drive is impacting local communities, are there any plans to allocate funds to support social causes? | Can you provide an update on the CJP protest and its potential implications on the current political landscape, particularly in regards to charitable organizations? | How do you think the recent developments in the Ram Mandir donation campaign will influence philanthropic efforts in India, especially for charities focused on education and healthcare?</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Aaj Tak Breaking News LIVE | Current Affairs News | CJP Protest | Headlines | Ram Mandir Donation Aaj Tak LIVE – International ...</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>2026-07-21T12:30:00Z</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=7rhl6BGcLUA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>WE HAVE YOUR 6 JULY FUNDRAISING FOR REGIMENT is in full swing!!</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>65</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>gamers</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>gaming</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>How does the Spearhead update impact the gameplay experience for Regiment players, and will the fundraising campaign offer exclusive in-game content? | What's the current progress on the WE HAVE YOUR 6 JULY FUNDRAISING campaign, and are there any specific charity initiatives that RegimentGG is supporting this month? | Will the Gray Zone Warfare 0.4 update include any new features that allow players to create custom charity events or tournaments within the game, similar to what we've seen in other gaming communities?</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>LIVE NOW – Gray Zone Warfare 0.4 “SPEARHEAD” UPDATE!! ​ ⁨@madfingergames⁩ ⁨@RegimentGG⁩ The battlefield just ...</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2026-07-21T00:06:27Z</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=d1TEM_LuSbo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Skyview - West of Frontier Ag Inc - Goodland, KS</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>30</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Farmers, Agricultural Professionals, or Local Community Members</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>I'm curious to know if Frontier Ag Inc has considered partnering with local charities to use this skyview service for environmental monitoring or disaster response efforts? | How does the community service aspect of this skyview project align with Frontier Ag Inc's overall corporate social responsibility goals, particularly in terms of supporting local Kansas initiatives? | Are there any plans to use the footage from this skyview service to support educational programs or workshops, potentially in partnership with local non-profits or charities focused on agriculture or conservation?</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>View of the skies west of Frontier Ag Inc in Goodland Kansas. A community service from Frontier Ag Inc. https://frontieraginc.com/</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2025-12-17T05:45:00Z</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=XjuKPeQx2V0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Skyview - East of Frontier Ag Inc - Goodland, KS</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>30</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Farmers, Agricultural Professionals, or Local Community Members</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>I'm curious to know if Frontier Ag Inc has considered partnering with local charities to utilize this skyview for environmental monitoring or conservation efforts? | How does the community service aspect of this skyview project align with Frontier Ag Inc's overall corporate social responsibility initiatives? | Are there any plans to use this skyview to support disaster relief or emergency response efforts in the Goodland, KS area, potentially in collaboration with local non-profits?</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>View of the skies east of Frontier Ag Inc in Goodland Kansas. A community service from Frontier Ag Inc. https://frontieraginc.com/</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2025-12-17T05:50:00Z</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=PrqfpZq4ERI</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Skyview - South of Frontier Ag Inc - Goodland, KS</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>30</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Farmers, Agricultural professionals, or individuals interested in weather conditions</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>I'm curious to know if the community service initiative by Frontier Ag Inc has led to any notable improvements in local air quality monitoring, given the proximity to agricultural areas? | Has Frontier Ag Inc considered partnering with local charities or environmental groups to further amplify the impact of their community service efforts in Goodland, KS? | Are there any plans to expand the skyview monitoring to other locations within Kansas, potentially in collaboration with regional conservation organizations?</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>View of the skies south of Frontier Ag Inc in Goodland Kansas. A community service from Frontier Ag Inc. https://frontieraginc.com/</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2025-12-17T05:50:00Z</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=xU7UDBXiAwA</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Skyview - North of Frontier Ag Inc - Goodland, KS</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>30</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Farmers, Agricultural enthusiasts</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>I'm curious to know if Frontier Ag Inc has considered partnering with local charities to use this skyview service for environmental monitoring or conservation efforts? | How does the community service aspect of this skyview project align with Frontier Ag Inc's overall corporate social responsibility goals, particularly in the Goodland Kansas area? | Are there any plans to use the footage from this skyview service to support educational initiatives or fundraising campaigns for local charities, such as those focused on agriculture or rural development?</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>View of the skies north of Frontier Ag Inc in Goodland Kansas. A community service from Frontier Ag Inc. https://frontieraginc.com/</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2025-12-17T05:50:00Z</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=70YcImm96ws</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Skyview - South of Frontier Ag Inc - Quinter, KS</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>30</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Farmers, Agricultural Professionals, or Local Community Members</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>I'm curious to know if the community service initiative by Frontier Ag Inc has led to any notable improvements in local weather monitoring or emergency response systems in Quinter, KS? | How does the view from Skyview contribute to the overall mission of Frontier Ag Inc, and are there plans to expand this community service to other locations? | Are there any partnerships or collaborations with local charities or organizations that Frontier Ag Inc is involved with, and how can viewers support these efforts?</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>View of the skies south of Frontier Ag Inc in Quinter Kansas. A community service from Frontier Ag Inc. https://frontieraginc.com/</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-03-13T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=NIGhF4jUja0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Skyview - West of Frontier Ag Inc - Quinter, KS</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>30</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Farmers, Agricultural Professionals, or Local Community Members</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>I'm curious to know if Frontier Ag Inc has considered partnering with local charities to use this skyview service for environmental monitoring or conservation efforts? | How does the community service aspect of this skyview initiative align with Frontier Ag Inc's overall corporate social responsibility goals, particularly in terms of supporting local Kansas communities? | Are there any plans to use the data collected from this skyview service to support precision agriculture practices or inform decision-making for sustainable farming methods in the Quinter area?</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>View of the skies west of Frontier Ag Inc in Quinter Kansas. A community service from Frontier Ag Inc. https://frontieraginc.com/</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-03-13T19:45:00Z</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=VbHOKakFTqo</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Skyview - North of Frontier Ag Inc - Quinter, KS</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>30</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Local farmer or agriculture enthusiast</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>I'm curious to know if the community service aspect of this project includes any educational programs for local kids about agriculture and sustainability, perhaps in partnership with a charity? | How does Frontier Ag Inc plan to utilize this skyview service to support local farmers and ranchers, and are there any plans to expand this initiative to other locations? | Are there any opportunities for viewers to get involved and support the community service efforts of Frontier Ag Inc, such as volunteering or donating to a related charity?</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>View of the skies north of Frontier Ag Inc in Quinter Kansas. A community service from Frontier Ag Inc. https://frontieraginc.com/</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-03-13T20:40:00Z</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Sf7OzR_oVqs</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>How Philanthropy Can Feed Business</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>89</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Entrepreneurs, Business Owners, Philanthropists</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Non-Profit, Business</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Wafa, can you share an example of a company that's successfully integrated philanthropy into their business model, and how it's impacted their bottom line? | I'm curious to know more about the role of CSR in driving business growth - are there any specific industries where philanthropy has been a key differentiator? | How do you think businesses can balance the desire to 'do good' with the need to measure ROI on their philanthropic efforts, and what metrics should they be tracking?</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>What happens when philanthropy does more than fund programs—and starts helping businesses grow? Wafa Dinaro, Executive ...</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-07-21T16:27:04Z</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=JtGPVv218_s</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>🔴LIVE: Trading Bot Scalping✅Giving Code Away For FREE✅</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>75</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Individual traders or investors interested in day trading and automated trading bots</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Finance/Trading</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Curious to know how you handle slippage when scaling up your trading bot, especially during high-volatility moments in the S&amp;P 500 futures | What's your strategy for avoiding overfitting in the bot's code, and are you using any specific backtesting methods to validate its performance? | Have you considered donating a portion of your profits to charity once you reach your $100000 goal, potentially using your platform to raise awareness for a cause?</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>I live day trade S&amp;P 500 futures with the goal of reaching $100000 in profit. Sharing my journey in real-time with full transparency ...</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-07-21T16:16:16Z</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=LwTFHMRd5Jc</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Giving backshots for the greater good</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>75</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Young adults or teenagers interested in gaming or streaming content</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Gaming or Entertainment</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>How do you think 'backshots for the greater good' can be applied in a charity setting, particularly for fundraising events? | I'm curious to know if there are any specific strategies for maximizing the impact of backshots in charity work, such as partnering with influencers? | Can you share an example of a successful charity campaign that utilized backshots to raise awareness and drive donations?</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>You Should Subscribe for more.</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-07-21T16:21:59Z</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=sEYC6fl6UfA</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
+      <c r="O57" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refresh generated caches and data artifacts
Updates runtime-generated outputs after a livestream analysis run, including Python bytecode caches, SQLite/DB data files, the Excel export, and appended token usage records.
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O93"/>
+  <dimension ref="A1:O113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4599,18 +4599,1001 @@
           <t>YouTube</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
           <t>https://youtube.com/watch?v=iEHU8Kiybdo</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="inlineStr"/>
-      <c r="O93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Rose#1 New Student Charity Member</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>90</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Philanthropist</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>What's the average financial burden that these students are facing, and how will the donated funds be allocated to support their college expenses? | Are there any specific college-related costs that this charity is focusing on, such as tuition, textbooks, or living expenses? | How will the charity ensure transparency and accountability in the distribution of funds to the students, and are there any plans for long-term support or mentorship programs?</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>this channel for charity student to helping they're financial in collenge pls help them thank you PAYPAL :charityphil26@gmail.com.</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:01:03Z</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Vuu7R_wNNgQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>NEW DONATION GAME?! I&amp;#39;M BACK DONATING ROBUX TO LIVE VIEWERS 🔴 LIVE 🔴</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>90</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Young adults and teenagers</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>How do you decide who to donate Robux to during the livestream, is it completely random or are there specific criteria? | I've noticed some viewers are sharing their Robux wishlists in the Discord server, do you take those into consideration when donating? | Are you planning on doing any charity fundraisers or collaborations with other streamers in the future, perhaps for a specific Robux-driven charity event?</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>JOIN UP AND GET A LAUGH OR TWO :D Discord server: https://discord.gg/UDxuJfESc Game link: ...</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:38:34Z</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=APismqX3YlI</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Trying to get a $5 Donation or any Donation</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>90</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Donor</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Non-Profit</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>I'm curious, have you considered partnering with a charity to amplify the impact of these $5 donations, perhaps a local food bank or education initiative? | For those donating via Venmo, will there be any public acknowledgement or leaderboard to encourage others to contribute, similar to a charity marathon? | Are there any plans to offer incentives or matching donations for certain milestones, like a $100 or $500 target, to motivate viewers to give?</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Donat apple pay:droninja3@gmail.com venmo: https://venmo.com/u/Droninja.</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:51:59Z</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=OFi3N-EGctQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>project live !  colleting 50 gift rasing and adding people in donation central #roblox #donating</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>85</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Gamers and philanthropists</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>How are you planning to track the 50 gift raisings in Donation Central, is there a specific leaderboard or dashboard you're using? | I'm curious, what kind of items are being donated in Roblox and how will they be distributed to those in need? | Are there any plans to collaborate with other Roblox streamers or charities to amplify the donation efforts and reach a wider audience?</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>This stream is created with #PRISMLiveStudio.</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-07-29T06:10:15Z</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=0_6pPoU3EPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Playing Donation Central Raising Stream</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>90</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>philanthropist</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>gaming</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>What's the average donor retention rate you've seen in charity streams like Donation Central, and how do you think we can improve it? | I'm curious about the tech behind Donation Central - are you using any specific plugins or integrations to facilitate donations and track engagement? | How do you handle transparency and accountability in charity streams, ensuring that donors know exactly where their funds are going and what impact they're having?</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-07-29T06:14:11Z</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=YBpFBT9M9TU</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>VR chat fishing and chilling friends only !charity !stackup !calltoarm</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>80</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Gamers and donors</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>How does the Stack Up charity initiative plan to allocate the funds raised from this VR chat event, and what specific causes will they be supporting? | I'd love to know more about the Discord server's role in organizing this charity event - are there any specific channels or resources available for attendees to get involved? | Will there be any opportunities for viewers to participate in the VR chat fishing and chilling activities, or are they primarily for entertainment while we support the charity drive?</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://discord.gg/nQtrHEy https://www.twitch.tv/kibathebarbarian https://tiltify.com/@kibathebarbarian/kibathebarbarian Join our ...</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-07-29T00:57:48Z</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=ftgdaKQOZuI</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>🔴Charity Gayle Christian Worship Songs 2025 - Best Praise and Worship Songs Of Charity Gayle</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>90</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Devout Christian</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Non-Profit</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>I'm curious to know if Charity Gayle's worship songs will be featured in any upcoming charity events or fundraisers, potentially raising awareness for social causes? | What's the story behind Charity Gayle's most popular praise song - is there a specific inspiration or experience that drove its creation? | Are there any plans to collaborate with other Christian worship artists or bands to create a charity album or single, with proceeds going to a notable cause?</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Charity Gayle Christian Worship Songs 2025 - Best Praise and Worship Songs Of Charity Gayle ▻Our main goal is to create a ...</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-07-28T07:25:00Z</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=v2xlAaUvceI</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>CommuniKitty CATURDAY! Cutie Cats ~ Free Games: !FOOD !Charity !Throne !Tip !YT !Kick CatGPT: Mother</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>80</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Animal Lover</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>How does the charity aspect of CommuniKitty CATURDAY work, are there specific organizations that benefit from the !Charity donations? | I'm curious about the !Throne game, is it a popular choice among viewers and does it have any impact on the charity donations throughout the stream? | Are there any plans to collaborate with other charity streams or organizations, perhaps through the !Discord hub, to amplify the fundraising efforts?</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Made with Restream. Livestream on 30+ platforms at once via https://restream.io VOTE !Angel Art: !Discord | !Hubby !Dix !Tip !</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-07-29T04:28:18Z</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=eAv612q4p5A</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Welcome back Glasses 🤓 Fundraiser Cash App 925Rucas</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>90</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Donor</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Non-Profit</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>How does the Glasses fundraiser plan to utilize the Cash App donations, specifically with the code 925Rucas, to support their charitable causes? | Can you share some insights on the impact of using Cash App for fundraising, like the 925Rucas campaign, in terms of donor engagement and retention for charity events? | What kind of transparency and updates can donors expect regarding the allocation of funds raised through the 925Rucas Cash App code, and how will it be used to benefit the charity?</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-07-29T05:55:31Z</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=ghCzZTmrGBk</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>live with mummy charity 💕 good morning my besties 💗 join my live</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>80</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Philanthropic Young Adult</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Non-Profit</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Love the charity focus today, Mummy! What inspired you to partner with this particular organization? | How do you plan to use the momentum from a viral video to drive donations and support for your chosen charity? | Will you be sharing any updates on the charity's current projects or initiatives that we can get involved with?</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>youtube #viralvideo.</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-07-29T06:03:42Z</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=LOLN_PqB_e4</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>NOVA TERMINATOR MODE! | Warzone Mayhem | Charity Stream  Can We Raise £5,000 For The Kids?</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>90</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>gamers and philanthropists</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>gaming</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>How's the donations tracker looking so far, are we on pace to hit that £5,000 goal for the kids by the end of the stream? | What's the plan for the Warzone gameplay, are you focusing on plunder or battle royale mode to maximize entertainment value for donors? | Will there be any special charity-themed gaming challenges or incentives for viewers to contribute during the stream, like a 'donate-to-lose' or 'donate-to-win' segment?</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>LIVE NOW:Tonight we're dropping into Call of Duty: Warzone to have some fun while raising money for an amazing cause.</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>2026-07-28T19:14:23Z</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=4lmMl9pJyFs</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>🔴Live | PLS Donate &amp;amp; Donate Plus | Donating ROBUX To Fans! #roblox #robux #donateplus #plsdonate</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>90</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Gamers, Roblox enthusiasts</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>How do you handle ROBUX distribution to ensure fairness among fans, especially with the new Donate Plus system? | What's the criteria for selecting winners for the ROBUX giveaways, is it based on donation amount or random selection? | Have you considered partnering with Roblox game devs to create charity-themed games that integrate with Donate Plus for a good cause?</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Join The New Dono Game! Donate Plus!! https://www.roblox.com/games/77403470693847/Donate-Plus ROBUX GIVEAWAYS ...</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-07-29T04:01:05Z</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=_f5MJnFuyJE</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Streaming until I hit 500 subs and get my very first donation!</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>80</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>gamer/streamer</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>entertainment</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>What's the plan for the donation once you hit the 500 sub goal - will it be going to a specific charity or cause? | How do you think the energy of the stream will change once you reach your donation milestone - will you be doing anything special to celebrate? | Are you considering partnering with a charity for future streams, maybe doing a fundraiser or something similar to give back to the community?</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Have some popcorn, snacks with you to fully enjoy this cinema stream Don't forget to comments, Like &amp; subscribe or there will be ...</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-07-28T00:26:04Z</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=j0E369VHZN0</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Giving up is not an option!!</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>75</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Individuals interested in financial education</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Education/Finance</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>What strategies can be applied to maintain perseverance in the face of regulatory hurdles, like those from SEBI, when working towards a charitable cause? | How do you think the educational content on this channel can be leveraged to support fundraising efforts for charities, particularly in the context of financial literacy? | Can you discuss any personal anecdotes or case studies where persistence, as emphasized in the title, led to a successful charitable initiative or campaign?</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>This channel is only for education purposes!! we are not SEBI registered.</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-07-29T03:43:57Z</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=do5Tl2QXM_A</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>GIVING AWAY ADMIN TREADMILL Roblox +1 Speed Keyboard Escape LIVE! #roblox  #trending  #fyp</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>75</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Young adults and teenagers</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>How does the +1 Speed Keyboard Escape impact gameplay, especially in admin treadmill Roblox? | Are you considering donating to a charity from the proceeds of the viral livestream, maybe something related to gaming communities? | Can you share any tips on how to optimize the Roblox experience with the given keyboard setup for a seamless livestream?</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>fyp #funny #foryoupage #live #livestream #viral #trending #shorts #roblox.</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-07-29T03:28:32Z</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=-devLYrSOB4</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>🔴 MARVEL RIVALS RANKED! 🔴 WE&amp;#39;RE NOT GIVING UP!!</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>75</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Gamers</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>What's the reasoning behind ranking Spider-Man above Doctor Strange, considering their recent performances in the MCU? | How do you think the rankings would change if we factored in the characters' abilities in a team-up scenario, like the Avengers? | Curious to know if you've considered creating a separate ranking for villains - would be interesting to see how Thanos stacks up against other notable Marvel baddies</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-07-29T02:09:30Z</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=9EvUM9nkE5c</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>$1,775 to Talk to a Minister: Ottawa&amp;#39;s Fundraising Hypocrisy Exposed (LIVE) | Famelee TV</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>80</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Socially Conscious Individual</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Non-Profit</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>I'd love to know more about the specifics of Ottawa's fundraising laws and how they're being exploited - are there any particular loopholes that allow ministers to charge exorbitant fees for access? | How does this fundraising hypocrisy impact charitable organizations, like the ones I work with, who rely on government grants and support? | Can Riya and Sam discuss potential solutions to increase transparency in political fundraising, such as implementing stricter disclosure laws or donation caps?</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Riya and Sam are back — and this time they're roasting Ottawa's favourite pastime: political fundraising hypocrisy. From Mark ...</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-07-28T22:03:36Z</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=JqYsfd1d7RQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>🔴 PLS DONATE LIVE GIVEAWAY | GIVING ROBUX TO VIEWERS! (Roblox Live) 💸</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>90</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Gamers, particularly Roblox players</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>How do you decide who to donate ROBUX to first in the PLS DONATE LIVE game mode? | Are you donating ROBUX to viewers who are actively participating in the stream, like commenting or engaging with the chat? | Do you think the PLS DONATE LIVE feature could be used to raise awareness or funds for real-life charities, similar to charity streams on other platforms?</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>In this stream I am playing PLS DONATE LIVE donating ROBUX to EVERYONE. I'll be going around donating to everyone in "PLS ...</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-03-23T13:00:00Z</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=khu5WMfmpYQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ABP Ganga LIVE: Pune Murder Case | Lucknow Fire |Ram Mandir Donation | Mumbai Monsoon |Bharat Tiwari</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>100</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>General Audience</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>News/Media</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>What's the latest update on the Ram Mandir donation drive and how can individuals contribute to this cause, especially in the context of charitable giving? | Bharat Tiwari, can you shed some light on how the recent Lucknow fire incident has affected local charities and what relief efforts are being made? | How do you think the current monsoon situation in Mumbai will impact charitable organizations' ability to provide aid and support to those in need?</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>ABP Ganga 24x7 LIVE: Pune Murder Case | Lucknow Fire |Ram Mandir Donation | Mumbai Monsoon |Bharat Tiwari हर बार ...</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>2026-03-27T07:04:15Z</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=EjvJGfo7RbY</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>(REAL) 🔴Pls Donate Robux Giveaway Live | Giving Robux In Pls Donate Live (Roblox Robux Giveaway)</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>80</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Roblox players</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>How do you plan to use the donated Robux to support charitable causes within the Roblox community? | What's the most creative way you've seen a Roblox user utilize their donated Robux to give back to others? | Will you be partnering with any specific Roblox groups or charities for this giveaway, or is it more of an individual effort?</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>(REAL) Pls Donate Robux Giveaway Live | Giving Robux In Pls Donate Live (Roblox Robux Giveaway) #plsdonate ...</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>2026-06-15T22:10:00Z</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=n9U4z1JO824</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr"/>
+      <c r="L113" t="inlineStr"/>
+      <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
+      <c r="O113" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(dong): save all local benchmark evaluation, sentiment analysis and mac updates
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O401"/>
+  <dimension ref="A1:O442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18648,7 +18648,6 @@
           <t>General</t>
         </is>
       </c>
-      <c r="F401" t="inlineStr"/>
       <c r="G401" t="inlineStr">
         <is>
           <t>Meetup</t>
@@ -18665,16 +18664,1605 @@
           <t>Wed, Aug 5 · 7:00 PM ICT</t>
         </is>
       </c>
-      <c r="J401" t="inlineStr"/>
       <c r="K401" t="inlineStr">
         <is>
           <t>https://www.meetup.com/product-and-beyond-saigon/events/315505691/</t>
         </is>
       </c>
-      <c r="L401" t="inlineStr"/>
-      <c r="M401" t="inlineStr"/>
-      <c r="N401" t="inlineStr"/>
-      <c r="O401" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Charity Livestream for World Cancer Research Fund ...</t>
+        </is>
+      </c>
+      <c r="B402" t="n">
+        <v>63</v>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Organization Manager</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Charity</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>I'd love to know more about the specific research projects that will be funded by this charity livestream - are there any updates on the current fundraising goals?</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>Charity Livestream for World Cancer Research Fund ...
+YouTube · Colour with Claire
+&gt;1,8 N lượt xem: · 5 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Online charity &amp; causes conferences</t>
+        </is>
+      </c>
+      <c r="B403" t="n">
+        <v>71</v>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Organization Manager</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Charity</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Have you considered exploring the intersection of online conferences and grassroots fundraising strategies, especially for smaller charities with limited resources?</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>Online charity &amp; causes conferences
+Eventbrite
+https://www.eventbrite.com › online › charity-and-caus...</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>AI on Local Hardware: What Works, What Doesn’t, and Why (Guest Speaker)</t>
+        </is>
+      </c>
+      <c r="B404" t="n">
+        <v>12</v>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: Advanced AI Concepts-Ho Chi Minh City
+Attendees: </t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Sat, Aug 1 · 9:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/advanced-ai-concepts-ho-chi-minh-city/events/315687404/</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Diaspora Charity Webinar Tickets, Saturday 25 July</t>
+        </is>
+      </c>
+      <c r="B405" t="n">
+        <v>86</v>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Organization Manager</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Charity</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>How do you plan to measure the long-term impact of the charity initiatives supported by this webinar?</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>Diaspora Charity Webinar Tickets, Saturday 25 July
+Eventbrite
+https://www.eventbrite.com › diaspora...</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>IECF 2026 Policy &amp; Philanthropy Summit: All Together</t>
+        </is>
+      </c>
+      <c r="B406" t="n">
+        <v>86</v>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Recruiter, HR Manager</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>How do you see the intersection of policy and philanthropy influencing the allocation of funds for social impact initiatives in the next 2-3 years?</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>IECF 2026 Policy &amp; Philanthropy Summit: All Together
+Eventbrite
+https://www.eventbrite.com › iecf-202...</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026 Power of Philanthropy Summit</t>
+        </is>
+      </c>
+      <c r="B407" t="n">
+        <v>86</v>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Recruiter, HR Manager</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>How do you see the intersection of impact investing and traditional philanthropy evolving in the next 5 years, given the increasing focus on measurable outcomes?</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>2026 Power of Philanthropy Summit
+Eventbrite
+https://www.eventbrite.com › 2026-p...</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Philanthropy Summit: The Power of Community, Collaboration ...</t>
+        </is>
+      </c>
+      <c r="B408" t="n">
+        <v>90</v>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Non-profit professionals, Philanthropists</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Non-profit, Philanthropy</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>How do organizations balance community engagement with the need for measurable impact in their philanthropic efforts?</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>Philanthropy Summit: The Power of Community, Collaboration ...
+YouTube · The Non Profit Podcast Network
+&gt;40 lượt xem: · 8 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>International Aid events Online - Charity &amp; Causes</t>
+        </is>
+      </c>
+      <c r="B409" t="n">
+        <v>90</v>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Philanthropist</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Non-Profit</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>What strategies can organizations use to effectively measure the long-term impact of their online fundraising campaigns, especially when it comes to reaching underserved communities?</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>International Aid events Online - Charity &amp; Causes
+Eventbrite
+https://www.eventbrite.com › ... › Charity &amp; Causes</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>[Webinar] Making sense of 2026: Fundraising trends ...</t>
+        </is>
+      </c>
+      <c r="B410" t="n">
+        <v>80</v>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Fundraising professionals</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Non-profit fundraising</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>I'm curious to know how the shift towards digital fundraising will impact smaller non-profits with limited resources, and what strategies can be employed to level the playing field.</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>[Webinar] Making sense of 2026: Fundraising trends ...
+YouTube · Givebutter
+&gt;530 lượt xem: · 5 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Empowering Nonprofits: Fundraising in a Cashless World ...</t>
+        </is>
+      </c>
+      <c r="B411" t="n">
+        <v>95</v>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>non-profit organizations</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>non-profit</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>How do you recommend nonprofits balance the shift to digital fundraising with the need to maintain relationships with long-time donors who may be hesitant to adopt new payment methods?</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>Empowering Nonprofits: Fundraising in a Cashless World ...
+YouTube · Alterna Savings
+&gt;30 lượt xem: · 1 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Nonprofit Guide to Peer to Peer Fundraising 2026</t>
+        </is>
+      </c>
+      <c r="B412" t="n">
+        <v>95</v>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Non-profit organization</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Non-profit</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>Have you considered how to incentivize repeat donors to participate in P2P campaigns, and what strategies Mightycause has seen work best in encouraging this behavior?</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>Nonprofit Guide to Peer to Peer Fundraising 2026
+YouTube · Mightycause
+&gt;70 lượt xem: · 1 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Nonprofit holding 3rd annual fundraising event at Top Golf</t>
+        </is>
+      </c>
+      <c r="B413" t="n">
+        <v>95</v>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Philanthropist or supporter of non-profit organizations</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Non-profit</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>Have you considered partnering with local businesses like Top Golf to offer exclusive sponsorship packages for your fundraising event?</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>Nonprofit holding 3rd annual fundraising event at Top Golf
+YouTube · KRQE
+&gt;50 lượt xem: · 4 tháng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>[Webinar] Top strategies for mastering fundraising events</t>
+        </is>
+      </c>
+      <c r="B414" t="n">
+        <v>95</v>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Fundraising professionals, Non-profit event planners</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Non-profit</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>How do you balance the need for personal connections with donors at events while also ensuring a smooth and efficient check-in process for a large number of attendees?</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>[Webinar] Top strategies for mastering fundraising events
+YouTube · Givebutter
+&gt;940 lượt xem: · 2 năm trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>A Glimpse into Excellence: Global CSR &amp; Philanthropy ...</t>
+        </is>
+      </c>
+      <c r="B415" t="n">
+        <v>80</v>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Academic or University audience</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>How do you think CSR initiatives can effectively address the water scarcity issue in rural India, given the complex interplay between government policies, community engagement, and technological innovations?</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>A Glimpse into Excellence: Global CSR &amp; Philanthropy ...
+YouTube · Ganpat University, GUNI, Gujarat, India
+&gt;170 lượt xem: · 3 tuần trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>🌍 English Club at Myths Cafe – Every Tuesday!</t>
+        </is>
+      </c>
+      <c r="B416" t="n">
+        <v>23</v>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: HCMC - Myths community
+Attendees: </t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>Tue, Jul 21 · 7:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/hcmc-myths-community/events/315545540/</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Perfume &amp; Fragrance Craft Workshop</t>
+        </is>
+      </c>
+      <c r="B417" t="n">
+        <v>16</v>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: HCMC - Myths community
+Attendees: </t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>Fri, Jul 24 · 7:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/hcmc-myths-community/events/315545727/</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>🌍 English Club at Myths Cafe – Every Tuesday!</t>
+        </is>
+      </c>
+      <c r="B418" t="n">
+        <v>23</v>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>Meetup</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Organizer: HCMC - Myths community
+Attendees: </t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>Tue, Jul 28 · 7:00 PM ICT</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>https://www.meetup.com/hcmc-myths-community/events/315545541/</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Charities Aid Foundation</t>
+        </is>
+      </c>
+      <c r="B419" t="n">
+        <v>40</v>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Charity Webinar</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>I'd love to hear more about how CAF is addressing the issue of donor fatigue in the UK, given the current economic climate.</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>Charities Aid Foundation
+YouTube
+https://www.youtube.com › videos</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>🎮 LIVE Minecraft for Assam Flood Relief ❤️🌊 | Charity Stream | Help Assam</t>
+        </is>
+      </c>
+      <c r="B420" t="n">
+        <v>90</v>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Socially conscious gamer</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Non-profit</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>Thank you for streaming for a great cause! Every donation counts in helping those affected by the Assam floods.</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=KHEJdMItGbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>The Great LEGO London Challenge LIVE FOR CHARITY!</t>
+        </is>
+      </c>
+      <c r="B421" t="n">
+        <v>90</v>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Family-oriented, philanthropic individuals</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Exciting to see LEGO enthusiasts coming together for a great cause! What's your favorite LEGO creation?</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=eOgiZjCHZlI</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>🔴 LIVE NOW | Meru County  Join us as we follow the Tharaka University 530 KM Charity Walk for the E</t>
+        </is>
+      </c>
+      <c r="B422" t="n">
+        <v>140</v>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>2026-08-04T17:07:57Z</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=B5Mx9I9uyMQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Diabetes Awareness &amp;amp; Fundraising Event Adelaide</t>
+        </is>
+      </c>
+      <c r="B423" t="n">
+        <v>135</v>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>LIVE NOW! We're Happy to bring you Here! Streaming live from The Palms Banquet Hall Adelaide, 5 Famechon Cres, Modbury ...</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>2025-02-08T11:11:42Z</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=dwmWxqfIbSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>TDC Australi Fundraising Event Melbourne</t>
+        </is>
+      </c>
+      <c r="B424" t="n">
+        <v>135</v>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>LIVE NOW! We're Happy to bring you Here Streaming live from Mulgrave Community Centre 355 Wellington Rd, Mulgrave VIC ...</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>2024-03-30T08:29:24Z</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=hVsl7RBQZUk</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>🔴[DC ] CHARITY WEDS DUNCAN [8/8/2026]</t>
+        </is>
+      </c>
+      <c r="B425" t="n">
+        <v>90</v>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>2026-08-08T07:42:44Z</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Z8MC_lXRbdQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Delma #21 student charity member</t>
+        </is>
+      </c>
+      <c r="B426" t="n">
+        <v>90</v>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>this channel for charity student to helping they're financial in collenge pls help them thank you PAYPAL :charityphil26@gmail.com.</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>2026-08-08T06:01:44Z</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=suYrAr1shRc</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Flood relief charity stream Assam</t>
+        </is>
+      </c>
+      <c r="B427" t="n">
+        <v>80</v>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>Flood relief charity stream Assam.</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>2026-08-08T10:01:59Z</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=bzgsGfgnkHQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>เตะเพื่อน้อง Counterpain Charity Cup 4 เส้าการกุศล</t>
+        </is>
+      </c>
+      <c r="B428" t="n">
+        <v>80</v>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>เตะเพื่อน้อง Counterpain Charity Cup 4 เส้าการกุศล VIP เมืองกาญจน์เวชภัณฑ์ พบ KING BULL FC VIP กาญจนบุรี พบ บอยท่าพระจันทร์ FC ...</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>2026-08-08T09:16:00Z</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Z1OhnhuwMqQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>LEY 75 NEW STUDENT CHARITY MEMBER</t>
+        </is>
+      </c>
+      <c r="B429" t="n">
+        <v>80</v>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>LIVE , DANCING,MUSIC, STUDENT LIVE STREAMER TO HELP THEY'RE STUDY PLS HELP US THANK YOU SO MUCH.</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>2026-08-08T09:15:20Z</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=3NXu-XjjElU</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Environmental Volunteers Live Stream</t>
+        </is>
+      </c>
+      <c r="B430" t="n">
+        <v>77</v>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>2026-08-07T18:29:54Z</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=o4sS0OJO75o</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Aaj Ki Taza Khabren LIVE: Weather Update | Ranchi Student Protest  | Badrinath Donation Scam</t>
+        </is>
+      </c>
+      <c r="B431" t="n">
+        <v>75</v>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>Aaj Ki Taza Khabren LIVE: Weather Update | Ranchi Student Protest | Badrinath Donation Scam दिल्ली में टूटा 15 ...</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>2026-08-08T01:00:23Z</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=oWf1_OqLwsg</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>(REAL) 🔴 PLS DONATE LIVE | GIVING ROBUX TO VIEWERS! (Roblox Giveaway) 💰</t>
+        </is>
+      </c>
+      <c r="B432" t="n">
+        <v>75</v>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>freerobux #plsdonate #robux #freerobux #plsdonate #robux In this stream I am playing PLS DONATE LIVE donating ROBUX to ...</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>2026-06-15T22:18:32Z</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=a6ju_zwS_fY</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>🔴 #HELLDIVERS2 : Giving em HELL on HELLMIRE</t>
+        </is>
+      </c>
+      <c r="B433" t="n">
+        <v>75</v>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>Support me at Kofi: https://ko-fi.com/tana_sukke/goal?g=0 . Follow me on other platforms .</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>2026-08-08T03:03:17Z</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=X5Gvog88-rU</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>🔴 Giving Seeds to Every Viewer LIVE! (Grow A Garden 2 Live) Free Pets Giveaway</t>
+        </is>
+      </c>
+      <c r="B434" t="n">
+        <v>75</v>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>Welcome to the stream! Today I am giving away Seeds &amp; Pets to Every Viewer LIVE! This is the biggest Grow A Garden 2 ...</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>2026-07-22T23:03:43Z</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=wtfxUyPWE_M</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Live on Donut Smp |Rating bases,giving money|loot drop|JOIN NOW!!!</t>
+        </is>
+      </c>
+      <c r="B435" t="n">
+        <v>75</v>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>LIVE ON DONUT SMP!** Today we're going all out on **Donut SMP**! Rating YOUR bases Giving away money Loot ...</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>2026-08-08T09:28:10Z</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=IIXHj4Ej8zI</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Fortnite Playing w/ subs &amp;amp; giving away sprites| USE CODE: NXBYT</t>
+        </is>
+      </c>
+      <c r="B436" t="n">
+        <v>75</v>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>2026-08-08T07:00:41Z</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=YU6u754KeXs</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>🔴BLOX FRUITS PERM DRAGON FRUIT GIVEAWAY | GIVING AWAY FREE FRUITS LIVE!</t>
+        </is>
+      </c>
+      <c r="B437" t="n">
+        <v>75</v>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>BLOX FRUITS PERM DRAGON FRUIT GIVEAWAY! #bloxfruitslive #bloxfruitslive #bloxfruitsroblox #bloxfruitsgiveaway ...</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>2026-01-06T06:20:09Z</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=L3hgmgoMqQQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>I&amp;#39;m streaming until I beat EVERY Sonic Game... please help. (DAY 3)</t>
+        </is>
+      </c>
+      <c r="B438" t="n">
+        <v>65</v>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>DONATE 2 CHARITY HERE: https://tilt.fyi/6VEystKlyl LEADERBOARD: https://tilt.fyi/UZ2WslUx1B Donation Incentives: $50 NUKE ...</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>2026-08-07T20:40:37Z</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=l8weFEfHUm8</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>FINAL Pokopia Bubbly Basin CHARITY Stream, @SU2C</t>
+        </is>
+      </c>
+      <c r="B439" t="n">
+        <v>90</v>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Gamers and philanthropists</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>Thank you for supporting a great cause! Your donations will help make a difference in the fight against cancer.</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=2Yu86v3LGLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>EP 25. Sulphur and Testing [!hardmode 25x] | Extra Life Charity Stream</t>
+        </is>
+      </c>
+      <c r="B440" t="n">
+        <v>90</v>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Gamers and philanthropists</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>Thanks for streaming for a great cause! Good luck with your gaming challenges and I hope you reach your charity goals.</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=WvA2AH7u3KQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>mummy charity ufomba is live!</t>
+        </is>
+      </c>
+      <c r="B441" t="n">
+        <v>90</v>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Philanthropist</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Non-Profit</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>Thank you for supporting a great cause! What will the donations from this livestream be used for?</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=7uGPoDc90T4</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>The 1st Annual Misti Media Book Fair</t>
+        </is>
+      </c>
+      <c r="B442" t="n">
+        <v>60</v>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Book lovers, Students, Educators</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Education/Entertainment</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>Excited for the book fair! Will any proceeds be going to support a charitable cause?</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr"/>
+      <c r="I442" t="inlineStr"/>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=wub4C1yzbKY</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr"/>
+      <c r="L442" t="inlineStr"/>
+      <c r="M442" t="inlineStr"/>
+      <c r="N442" t="inlineStr"/>
+      <c r="O442" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refactor AI scoring and cleanup legacy modules
This commit replaces the legacy rule-based relevance flow with a unified ML/NLP scoring pipeline. Spam detection and relevance scoring are now centralized in ai/spam_classifier.py, event classification falls back to semantic scoring when LLMs are unavailable, and goal/topic expansion code was updated to use the new flow. It also removes obsolete legacy files (gemini.py, summarize.py, train_supercharged_spam_model.py, relevance_filter.py), adds project documentation, and refreshes cached data/log artifacts to match the new system behavior.
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livestreams" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Livestreams" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O130"/>
+  <dimension ref="A1:O137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6442,6 +6442,188 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>🔥MENHELYEN JÁRTAM🔥PÉNTEKTŐL VASÁRNAPIG CHARITY STREAM🔥 I JUST CHATTING</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>90</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=rpckPiTWTSU</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>monday morning hardcore [ minecraft | bedrock | hardcore | !legends ] !charity</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>80</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Bc4hyMI5Jn4</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>LEGO Charizard Build Livestream for Charity!</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>80</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=O4O7wik4ynk</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>satkartar satsang ghar charitable society is live!</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>56</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=uqX2-mzcmSQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Jesus Protects You, Eliminates Evil &amp; Brings Healing, Peace &amp; Miracles Into Your Life Instantly</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>41</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=uDgzWqNstjI</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Beaver Cam</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>34</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=zkTaY9OQM2A</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>WORDFEST 2026 || DAY 2|| EVENING SERVICE || REV MARTIN || TILL NO. 837898 || 10.08.026</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>34</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=lrXDSoEvtBo</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr"/>
+      <c r="L137" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Auto-infer event region, enrich channel metadata with niche keywords, fix DateTime/encoding bugs, add 10 US test channels
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O130"/>
+  <dimension ref="A1:O204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6442,6 +6442,3387 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Trưa Mùng11Tháng7Âm Mở Kinh CầuAn Mẹ Rất LinhỨng Hộ Trì Tiền Vô Như Nước MuaBán Đắt Đỏ Vạn Sự Như Ý!</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>190</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Small business owners, retailers, online sellers, entrepreneurs, and individuals engaged in trade who seek spiritual blessings for financial prosperity and booming sales.</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Commerce &amp; Spirituality</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Thật đúng dịp Mùng 11 Tháng 7 Âm này, con cũng đang cầu Mẹ phù hộ cho công việc kinh doanh cuối năm được thuận lợi, hàng hóa đi nhanh ạ. | Nghe Kinh Mẹ xong cảm giác tâm an hẳn, hy vọng Mẹ sẽ hộ trì cho dòng tiền về dồi dào để các kế hoạch đầu tư sắp tới được hanh thông. | Mẹ linh ứng lắm ạ, con xin Mẹ che chở để team bán hàng của con luôn gặp khách tốt, chốt deal thành công, vạn sự như ý trong mọi giao dịch.</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Trưa Mùng11Tháng7Âm Mở Kinh CầuAn Mẹ Rất LinhỨng Hộ Trì Tiền Vô Như Nước MuaBán Đắt Đỏ Vạn Sự Như Ý!</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>2026-08-23T03:30:00Z</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=xjXrEU9AYy0</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>SALE LƯƠNG VỀ</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>150</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Salary earners, value-conscious shoppers, typically employed individuals looking for discounts and deals, especially around payday.</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>E-commerce / Retail</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Chào ad, đợt 'Sale Lương Về' này sản phẩm chủ lực nào đang có ưu đãi tốt nhất mà ad muốn nhấn mạnh không ạ? | Thấy có link Shopee rồi, vậy khi mua qua link này mình có được áp dụng thêm mã giảm giá độc quyền nào cho livestream hoặc freeship không ạ? | Nếu muốn hỏi chi tiết hơn về chất liệu hoặc kích thước sản phẩm mà chưa thấy trên livestream, mình có thể inbox Zalo số 0985592206 để được tư vấn riêng không nhỉ?</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Dalo 0985592206 Link mua hàng sàn cam https://s.shopee.vn/40UvJkjS9I.</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>2026-08-23T01:48:47Z</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=41wE-UEXq38</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>[23.8] MIỀN BẮC TUNG DEAL- SĂN SALE ẦM ẦM</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>150</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Parents (primarily mothers) of infants/toddlers, value-conscious and looking for deals on essential baby items like diapers.</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Baby Products Retail</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Cho mình hỏi là ưu đãi giảm 42k khi mua 3 gói Tã quần Molfix Oxygen này có áp dụng cùng với mã giảm giá khác từ Concung không ạ? Đang định mua tích trữ cho bé. | Thấy chương trình là 'Miền Bắc Tung Deal', vậy các tỉnh khác ở miền Trung/Nam có thể săn deal Molfix này không hay chỉ áp dụng riêng cho khu vực miền Bắc thôi ạ? Muốn mua gấu bông cho bé quá. | Mấy chương trình 'săn sale ầm ầm' kiểu này trên Concung thường diễn ra theo định kỳ không nhỉ? Mình thấy deal tã Molfix Oxygen đợt này khá hời mà sợ bỏ lỡ các đợt sau.</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Xem ngay tại: https://concung.vn/qkewar Giảm 42.000đ khi mua 3 gói Tã quần Molfix Oxygen M/L/XL/XXL Tặng quà gấu bông ...</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>2026-08-23T01:00:52Z</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=agr1_xp1XCU</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>🔥 ROBLOX 🔴 | A VER QUE SALE! 🎯💀</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>85</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Children/Teenagers, Roblox players, casual gamers, seeking entertainment and gameplay content.</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Viendo la dinámica, me intriga saber: ¿qué estrategias de monetización has visto que funcionan mejor para creadores en Roblox *actualmente*, más allá de los game passes? ¿Crees que el engagement se traduce bien a ingresos directos? | Con tantas marcas mirando Roblox para el comercio, ¿qué tipo de integración de productos virtuales crees que realmente conecta con los jugadores? Es clave que no se sienta forzado para ambos lados. | Esa emoción de 'A VER QUE SALE' es clave. ¿Qué crees que hace Roblox *bien* para que los jugadores sigan descubriendo y se queden en nuevas experiencias? Esos patrones de retención son súper importantes.</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>XxThejuan96xX #envivo #gameplay -------------------------------------------------------------------------------- •• MIS REDES SOCIALES ...</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>2026-08-23T04:12:59Z</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=aku9qM7wVDw</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Rankeando en LoL de chill (sale mal)🦊</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>85</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Casual League of Legends players and viewers, young adults, individuals seeking lighthearted gaming entertainment, viewers of smaller or hobbyist streamers.</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Gaming, Live Streaming, Entertainment</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Cuando la ranked 'sale mal' de chill, ¿sientes que es más fácil recuperarte en la siguiente o te cuesta quitarte el tilt del mapa anterior? Es un balance complicado. | Para lo de 'no saber qué contenido hacer', ¿has pensado en grabar esos momentos épicos donde 'sale mal' y luego hacer un compilado? A veces esas risas conectan más que el gameplay perfecto. | Siempre me pregunto si el 'de chill' es una estrategia activa para no estresarse o si simplemente es el mood del momento. Y ese 🦊, ¿es por algún main champ o solo good vibes?</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Hago stream cada milenio. Ya no se que contenido hacer xd Timeline de partidas: 0:00 - Inicio (no me digas) ...</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>2026-08-23T03:49:47Z</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=afcXlDDQSA0</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>🔴 UN DÍA MÁS RATEANDO EN FORTNITE 🐀😂 | ¿HOY SALE VICTORIA? 🏆</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>85</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Fortnite players, gamers, couples who game together, viewers seeking casual and entertaining gameplay streams, audience interested in 'rat' style gameplay.</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Gaming</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Genial el 'modo rata' en acción. Pensando en optimización, ¿qué tan consistente les ha resultado esta estrategia para la victoria final en duos, comparado con un push más directo? | Cuando están en 'modo rata', ¿cómo evalúan el riesgo-recompensa de quedarse en un punto vs. hacer un movimiento arriesgado? Esa 'inversión' de tiempo para el endgame es clave. | Con el objetivo de la victoria hoy, y viendo el meta actual, ¿creen que el 'modo rata' ofrece un mejor 'retorno de inversión' de esfuerzo que una estrategia ultra-agresiva en duos?</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>LAS RATITAS SALIERON A RATEAR! Hoy toca Fortnite en pareja, jugando con mi polola y activando el MODO RATA al ...</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>2026-08-23T03:44:07Z</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=MpRDKkK2YMk</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>sale un codsito?? - Baty Reyes #codm</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>100</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Mobile gamers, Call of Duty: Mobile players, fans of Baty Reyes, individuals interested in casual gaming content.</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Gaming, Live Streaming</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Baty, qué onda con esa CBR4, ¿la sigues usando en ranked o ya te pasaste a la Kilo? Siento que la CBR es más consistente para rushear ahora. | Con el último update, ¿qué opinas de Crossfire en Dominio? A mí se me complica un montón si el otro equipo controla bien el edificio central para la B. | Siempre me cuesta un montón contra los snipers agresivos en BR. ¿Algún consejo para pushearles sin que me den un headshot al instante? ¿Depende mucho del perk?</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>codm #callofdutymobile #batyreyes.</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>2026-08-23T03:24:31Z</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=kQiF_QFJ0aA</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Tư vấn săn sale cơ bida môi ngày trên Live trym</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>95</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Billiard players, enthusiasts, or individuals looking to purchase billiard cues, especially those interested in finding daily deals or discounts through a livestream format.</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Billiards Equipment Retail, Sporting Goods, E-commerce</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Thanh Minh chia sẻ thêm xíu được không là mình tập trung săn sale các dòng cơ bida phổ biến hay có bất ngờ với những mẫu cao cấp trên livestream mỗi ngày ạ? | Với lịch livestream săn sale cơ bida mỗi ngày, Thanh Minh có mẹo nào để khách hàng dễ theo dõi và không bỏ lỡ các deal hot, đặc biệt với những ai muốn mua số lượng không? | Mình thấy địa chỉ xưởng ở Hiệp Bình Chánh, vậy Thanh Minh có thể bật mí quy trình kiểm tra chất lượng cơ bida trước mỗi phiên săn sale trên live không? Rất quan tâm về độ bền và giá trị đầu tư lâu dài.</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Billiards Thanh Minh ◅ Địa Chỉ Công Ty : 299 , Lê Hồng Phong , phường 2 , Quận 10 . Địa Chỉ Xưởng : Hiệp Bình Chánh , TP .</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>2026-08-23T03:00:21Z</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=yw4vr5LrSAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Y SI ME SALE UN ROJO❓#arenabreakoutinfinite</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>85</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Sorrelowski, si te sale un 'rojo', ¿cuál es tu estrategia principal? ¿Vas directo a por el high-risk/high-reward o intentas asegurar la extracción primero? | Pensando en lo del 'rojo', ¿hay alguna configuración de arma o tipo de munición específico que uses para maximizar tus chances contra ese tipo de encuentro, o prefieres ser más versátil? | Si consigues sacar un 'rojo' de la raid, ¿sientes que vale la pena el riesgo adicional para venderlo en el mercado o prefieres usarlo tú mismo para futuras incursiones de alto valor?</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>REDES SOCIALES ₪ ₪ ₪ ₪ ₪ ₪ ₪ ₪ ₪ ₪ https://www.youtube.com/@Sorrelowski https://www.tiktok.com/@sorrelowski ...</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-08-23T02:26:53Z</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=fC_QamIaI0Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Online Payday Sale</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>98</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>General consumers, employees with disposable income, individuals seeking deals and discounts around their payday.</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>E-commerce / Retail</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Curious if there are any specific bundle deals or loyalty program bonuses planned for this payday sale, especially for repeat customers looking to maximize value? | Will there be any specific payment gateway promotions or cash-back offers tied to certain banks during this online payday event? Sometimes those really make a difference for bigger purchases. | Wondering if there will be particular 'flash sale' windows or early bird access for some of the higher-demand items today? Always tricky to catch those on payday sales!</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-08-22T23:59:54Z</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=_qJX4MU346Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>23/8 Giam Can ngay 13(Mua lam vch)</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>85</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Individuals interested in health, fitness, and personal weight loss journeys; potentially consumers of health-related products.</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Health &amp; Wellness</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Thắng Đông Anh * Lịch stream: Ca sáng:8h-11h Ca chiều: 2r-5h Ca tối: flex * Thông tin của mình - FB cá nhân: ...</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-08-23T01:18:05Z</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=qppQT8ld4nA</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Can AI Really Read an Ultrasound? Watch MUA-AI Interpret Images in Real Time!</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>85</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>LIVE: Can AI Really Read an Ultrasound? Watch MUA-AI Interpret Images in Real Time!** Join **Medical Ultrasound Academy ...</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>2026-08-22T19:29:45Z</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=_X1ic4ZSK70</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Cổ Nhân Dạy - Dù Có Tiền Tỷ Cũng Đừng Mua 6 Thứ Này! Về Già Nhục Lắm</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>85</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>CHỈ CẦN DẬY LÚC 3 ĐẾN 5 GIỜ SÁNG, BẠN SẼ THAY ĐỔI CẢ CUỘC ĐỜI | TRIẾT LÝ CUỘC SỐNG | LỜI DẠY CỔ NHÂN.</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>2026-08-22T01:47:29Z</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=2e2xdDM_TTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>[Trực Tiếp] | MUA SẮM ONLINE - NGẬP TRÀN ƯU ĐÃI - ĐỘC QUYỀN TRÊN SCJ TV SHOPPING</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>85</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Chào mừng bạn đến với kênh mua sắm trực tiếp chính thức của SCJ TV SHOPPING trên YouTube! Giờ đây, bạn có thể xem ...</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>2026-08-19T13:02:44Z</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=0nlpfooY9lY</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>SỰ THẬT KINH HOÀNG TIỀN ĐIỆN NƯỚC: Dân Kêu Cứu Bác Tô Lâm, Bà Phương Hằng Vạch Trần Sự Thật!</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>85</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>SỰ THẬT KINH HOÀNG TIỀN ĐIỆN NƯỚC: Dân Kêu Cứu Bác Tô Lâm, Bà Phương Hằng Vạch Trần Sự Thật! #tiendien ...</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>2026-08-23T03:26:11Z</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=TZryfBt-PQU</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>🏆 GIẢI PICKLEBALL NỘI BỘ CLB KINH MÔN</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>85</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>GIẢI PICKLEBALL NỘI BỘ CLB KINH MÔN NGÀY THI ĐẤU: 23/ 08/ /2026. ĐỊA ĐIỂM: CỤM SÂN TRÚC LỘC PICKLEBALL.</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>2026-08-23T00:19:54Z</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=j3fqHxeKPqk</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>🔴 Kinh Di Giáo 24/7 | Lời Di Huấn Cuối Cùng Của Đức Phật • Tụng Kinh An Lạc • Thích Trí Bửu</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>85</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Kinh Di Giáo 24/7 là livestream tụng trì những lời di huấn cuối cùng của Đức Phật Thích Ca Mâu Ni trước khi Ngài nhập Niết-bàn.</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>2026-08-20T07:06:42Z</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=z8uHZqEU_k0</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>🔴Vu Lan Báo Hiếu Nghe Kinh Này Tỷ Lần Rơi Lệ, Báo Đáp Công Ơn Cha Mẹ</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>85</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>giacngochantam Nam mô Đại Hiếu Mục Kiền Liên Bồ Tát. Có những yêu thương trên đời, khi còn ở bên ta, ta cứ ngỡ đó là điều ...</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>2026-08-12T16:40:00Z</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=z-UcCMZfs7k</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Kinh Địa Tạng Trọn Bộ 🙏 Bài Kinh Linh Ứng Nhất – Giải Nghiệp, Gia Đạo Bình An</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>85</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Kinh Địa Tạng Trọn Bộ Bài Kinh Linh Ứng Nhất – Giải Nghiệp, Gia Đạo Bình An Nghe Kinh Địa Tạng Trọn Bộ giúp người nghe ...</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>2026-08-14T05:00:39Z</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=LB1AnepCIqo</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Tụng Kinh Dược Sư -  Nghe Mỗi Ngày Cầu Bình An , Hết Bệnh Hết Khổ, Tiêu Tai Giải Nạn | Kinh Tụng</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>85</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Sale
+Mua Bán
+Kinh Tế</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>KINH DƯỢC SƯ – Tụng Kinh Dược Sư - Nghe Mỗi Ngày Cầu Bình An, Tiêu Tai Giải Nạn, Hết Bệnh Hết Khổ Kinh Dược Sư là một ...</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>2026-08-16T10:10:00Z</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=8Bdsk-FID3U</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Business Growth TV 24/7 | Entrepreneurship, Leadership, Marketing &amp;amp; Small Business Success</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>340</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Small Business Owners, Entrepreneurs, Business Leaders, Marketing Professionals, Startup Founders</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Business Services / Consulting / Education / Marketing</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Hey team, when we're talking 'marketing for small business success,' what's a lesser-known strategy that significantly boosts enterprise value for a *potential sale*, not just daily lead gen? | Thinking about the 'leadership' aspect for growth: are there specific operational redundancies or 'owner-dependent' systems small businesses often neglect that really bite them when trying to scale or get acquired? | With 'real-world strategies' in mind, what's one key move a small business can make early on to build a truly *defensible* competitive moat, beyond just a unique product, that makes it an attractive acquisition target?</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Welcome to Business Growth TV 24/7, powered by The Prosperity Lounge — nonstop conversations, strategies and real-world ...</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>2026-08-15T17:13:27Z</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=svYQjgEnlGo</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Business Story of the Week 24/7 Live: Entrepreneurial Insights &amp;amp; Growth Mindset</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>200</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Entrepreneurs, small business owners, aspiring business leaders, professionals seeking growth, individuals interested in business strategy and personal development within a business context.</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Business, Entrepreneurship, Professional Development</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Curious, when focusing on entrepreneurial insights, how crucial is the *story behind the pivot* in building long-term brand resilience versus just showcasing the success? | Great to hear about growth mindset. What specific tactics do you recommend for founders to instill that *culture of iterative learning* across their early-stage team, especially when funding is tight? | For the business story you're covering, how did they initially *validate their problem-solution fit* without significant upfront capital? Always interested in those lean market entry strategies.</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Subscribe to the Channel: https://www.youtube.com/channel/UCX59Z1-L4LBe7-qKEz_-QzA/?sub_confirmation=1 Welcome to ...</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>2026-06-04T00:05:00Z</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=xXk768Fe064</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>RUQYAH DUA TO INCREASE RIZQ, BARAKAH, CUSTOMERS &amp;amp; SALES - CURE FOR BUSINESS STRUGGLES &amp;amp; PROBLEMS!</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>180</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Muslim business owners, entrepreneurs, or sales professionals seeking spiritual intervention and guidance from the Quran to resolve business struggles and boost sales and customers.</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Islamic Spiritual Services</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>For small business owners balancing daily operations, what's a realistic routine or frequency for implementing this Al Quran Ruqyah Shariah dua to see consistent growth in sales and barakah? | Many businesses face periods of stagnant customer acquisition or unexpected supply chain issues. Does the Ruqyah Shariah dua offer specific guidance for overcoming these particular 'business struggles and problems'? | It's powerful to think about increasing rizq and barakah. From a practical business standpoint, how have you seen the increase in barakah specifically translate into tangible improvements like better sales conversion rates or stronger customer loyalty?</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Most powerful Al Quran Ruqyah Shariah dua to increase rizq, barakah, customers and sales — delivering a powerful cure for ...</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>2026-08-22T20:25:00Z</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=kJ5N8YO-5I8</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>ENTREPRENEURSHIP SYMPOSIUM</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>145</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Aspiring entrepreneurs, small business owners, students interested in business, community members seeking business insights, individuals looking for tools and strategies for business growth.</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Entrepreneurship, Education, Faith-based Business</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>For founders eyeing quick scaling, what's a common mistake you see when trying to penetrate new markets, particularly around building out robust distribution channels or strategic local partnerships? | Love to hear the panel's perspective on identifying genuine market white space. What’s a signal you look for beyond just a perceived 'gap' – maybe something about unarticulated needs or technological leverage that indicates true breakthrough potential? | Beyond traditional VC, what are some underutilized funding strategies or non-dilutive capital sources that early-stage founders should really be exploring right now, especially those prioritizing sustainable revenue over hyper-growth?</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Welcome to University Seventh-day Adventist Church. We invoke rich blessings upon you from our Father in Heaven. Special ...</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>2026-08-23T06:58:52Z</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=xKkulrprVlE</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>TMP SUNDAY CELEBRATION SERVICE | ENTREPRENEURSHIP &amp;amp; INVESTMENT.</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>145</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Entrepreneurs, aspiring business owners, investors, individuals seeking financial growth and business insights.</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Business, Finance, Entrepreneurship</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Given the JHB context for this service, I'm curious if the discussion will touch on specific high-growth sectors or underserved markets where new entrepreneurs can make a significant impact and attract early investment. | On the investment side, I'm particularly interested in hearing strategies for securing seed funding within the local Strydom Park/JHB ecosystem. What are some key pitfalls to avoid when pitching for initial capital? | Considering this is a 'Celebration Service' focusing on Entrepreneurship &amp; Investment, I'm curious about the role of mentorship and community support networks in sustaining entrepreneurial growth beyond just securing capital. Any thoughts on fostering that in JHB?</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Dates: 23 AUGUST 2026 Venue: The Master's Place, 4 Commercial Avenue, Strydom Park, Johannesburg Guest Minister: Ms ...</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>2026-08-23T07:35:46Z</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=8PdW_zhyQ-c</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Blues Rock Entrepreneurs - Motivational Guitar Playlist Vision, Focus &amp;amp; Business Mindset - 4 Hours</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>145</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Blues/Rock Musicians or aspiring entrepreneurs seeking business guidance, motivation, and skill development for their music ventures.</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Music, Entrepreneurship, Self-help</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>How does the structure of a classic 12-bar blues, with its clear progression, offer a mental framework for entrepreneurs when they're mapping out a complex project or a long-term business vision? | This 'HollowSoul Blues' really gets into deep emotions. How do you suggest entrepreneurs channel that soulful intensity to maintain focus and conviction during a tough sales cycle or when facing market resistance? | For cultivating that 'focus' state, what specific elements of a slow blues guitar solo – maybe the bends or sustain – do you find most effective for sparking new ideas when I'm reviewing a P&amp;L or sketching out a new service offering?</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Welcome to HollowSoul Blues , a place where deep emotions, soulful guitars, slow blues, and timeless melodies come ...</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>2026-08-23T08:07:45Z</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=dIYqsvsN21c</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Business &amp;amp; Career (1st) Service-Dominion City Awoyaya| 23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>85</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Professionals, Entrepreneurs, Business Owners, Career-minded individuals seeking development and guidance.</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Religious (with Business &amp; Career focus)</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Given this is the *first* Business &amp; Career session for Service-Dominion City Awoyaya, I'm keen to hear what specific challenges local businesses here are currently navigating. Maybe talent acquisition or market access? | Intrigued by the 'Service-Dominion' part of the title. For those of us running businesses, how do you practically integrate those values into daily operations or strategic planning to drive growth within the community? | From a career perspective, especially for young professionals in Awoyaya, what's one non-obvious skill or networking strategy that could make a significant difference in their trajectory, given the local economic landscape?</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>2026-08-23T07:29:47Z</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=KnHaPBwSBGU</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>BUSINESS, CAREER &amp;amp; LEADERSHIP SERVICE II 23-08-2026 II 1ST SERVICE</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>85</v>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Professionals, entrepreneurs, and leaders seeking faith-based guidance for business and career growth, or individuals interested in spiritual development for their professional lives.</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Faith-based Professional Development/Ministry</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Rev. Abba, keen to hear your thoughts on navigating business growth targets while upholding deep spiritual integrity. How do we balance ambition with our 'wordalive' principles in competitive markets? | Many leaders struggle with long-term vision amidst daily pressures. What's a key spiritual discipline or 'wordalive' insight you recommend for maintaining that resilience and clarity? | For those of us aiming to expand our reach or overcome client acquisition challenges, what 'wordalive' perspective helps reframe these obstacles into opportunities for genuine purpose-driven impact?</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>LIKE, COMMENT &amp; SHARE #revgodwinabba #wordalive #LiveBroadcast #share #word #worship #praise #like #comment ...</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>2026-08-23T06:35:57Z</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=YpKPtpWcZ5Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>SUNDAY SERVICE || BUSINESS ACTIVATION CODE || TRADE FAIR || 23RD AUGUST, 2026.</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>95</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Small business owners, entrepreneurs, sales and marketing professionals, individuals seeking business growth and networking opportunities, those interested in faith-based business principles.</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Business Development, Entrepreneurship, Sales &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>SUNDAY SERVICE || BUSINESS ACTIVATION CODE || TRADE FAIR || 23RD AUGUST, 2026. MINISTERING: PST. OLAKUNLE ...</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>2026-08-23T06:36:53Z</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=jc5HX83q8vk</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>🔴 LIVE | No Doctor, Yet the Business Continued for 2 Years? | ASMITATVLIVE</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>85</v>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>General public, concerned citizens, viewers interested in public health and regulatory issues in the healthcare sector.</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Healthcare (News Reporting)</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>2 years is a long time for a nursing home to operate without proper medical staff. Were there any official inspections or audits during that period, or was it entirely off the radar until the raid? | Curious about the actual *business model* here. Without a doctor, how were patient cases being handled or billed, and what allowed them to maintain operations for so long from a financial standpoint? | Beyond the immediate shutdown post-raid, what are the longer-term consequences for the operators of this nursing home, especially concerning any fraudulent billing or patient safety violations over those two years?</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>LIVE | ଡାକ୍ତର ନାହାନ୍ତି, ତଥାପି ଚାଲିଥିଲା କାରବାର? ଚଢ଼ାଉ ପରେ ନର୍ସିଂହୋମ ...</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>2026-08-23T04:59:22Z</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=6kYCoxeDvRU</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>SPECIAL BUSINESS SERVICE TAGGED:OCCUPY WITH CHRIS EMMANUEL  23/8/2026</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>95</v>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Small business owners, aspiring entrepreneurs, real estate investors, individuals seeking business growth strategies, financial education seekers, direct sales professionals.</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Business Coaching, Entrepreneurship, Financial Services</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Chris, curious about the 'OCCUPY' strategy – for an SMB, what's typically the biggest *practical* hurdle in executing an aggressive market positioning without totally overstretching resources? Budget or team bandwidth usually? | Following up on 'OCCUPY,' once a business has established its foothold, how do you see them best fending off those inevitable competitive counter-moves for sustained market presence? It's a real balancing act. | Hi Chris, on the 'OCCUPY' concept, what's your go-to method for businesses to pinpoint those *truly* underserved market niches that are ready for aggressive capture, not just slow, incremental growth? That initial targeting feels key.</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>SPECIAL BUSINESS SERVICE TAGGED:OCCUPY WITH CHRIS EMMANUEL 23/8/2026 Connect with Chris Emmanuel: ...</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>2026-08-22T16:13:09Z</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=PGE45u68Ei4</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>💚 Music for Plants 🎵 Relaxing Plant Growth Music 24/7 🌱</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>85</v>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Sale 
+Business</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Welcome to Houseplant 101's relaxing music for plants stream — peaceful background music created for plant lovers, indoor ...</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>2026-08-23T08:32:31Z</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=s6mwUhK4IJ8</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Growth III || Youth Sunday Service || 23-08-26</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>85</v>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Church members, youth, individuals seeking spiritual worship</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Religious/Non-profit</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Growth III || Youth Sunday Service || 23-08-26 Join us as we worship . Church account Details: IE07AIBK93745223502061.</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>2026-08-23T08:01:57Z</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=FBbEzHT04qA</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>CELEBRATION SERVICE | PREPARE FOR GROWTH | PST GEORGE PAUL</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>85</v>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Sale 
+Business</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Welcome to our Sunday Celebration service We are truly grateful that you've joined us today. Wherever you're watching from, ...</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>2026-08-23T07:49:43Z</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=1GcLi5D3t9Q</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026 CONFERENCE SUNDAY || BELIEVER’S BALANCED GROWTH || REV&amp;#39;D NATHANIEL EKUNDAYO</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>85</v>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Sale 
+Business</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>AUGUST 23RD 2026.</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>2026-08-23T07:03:53Z</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=LYGni8mc3v0</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Podcast Replay | Socially Awkward Podcast: Hospitality Marketing</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>85</v>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Business Decision Maker</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Sales &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>This is a live replay of our best episodes, enjoy! Thanks for tuning in to Socially Awkward, the hospitality marketing podcast where ...</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>2026-08-19T19:54:43Z</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=o2-KSuMkE1U</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>live  gold trading everyday / XAUUSD &amp;amp; BTC/ Trading with My own strategy</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>85</v>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Sale 
+Business</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Admin only trade on demo accounts.This is just a video to learn about forex trading, and also not an invitation or advertisement to ...</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>2026-08-23T08:42:29Z</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=VTut1o_pF78</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Personal Branding Strategy  ala Rizqiani Putri</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>90</v>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Entrepreneurs, small business owners, freelancers, consultants, coaches, sales professionals, and anyone looking to leverage their personal brand to attract clients and drive sales for their business.</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Business Development, Marketing, Entrepreneurship, Coaching, Consulting</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>2026-08-23T08:17:53Z</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Z9jxZrcpNW0</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>LIVE Bitcoin &amp;amp; Gold Trading Strategy | 23 AUG | Market Analysis #gold #cryptotrading #livetrading</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>85</v>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Sale 
+Business</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>LIVE Bitcoin &amp; Gold (XAUUSD) Trading Strategy | Live Market Analysis #gold #cryptotrading #livetrading Welcome to today's LIVE ...</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>2026-08-23T07:34:21Z</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=eMfYfF7nY6A</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>map editor for grand strategy game in godot</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>85</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Sale 
+Business</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>https://rjljones.itch.io/grandfantasy.</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>2026-08-23T06:56:11Z</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=ItWP4hyio9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Super sale Dhmaka Rakhi special 🥳💥💥💥📲9050866606</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>76</v>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Sale
+Business</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Fu3chRBRlD0</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>CNBC TV18 24x7 LIVE: Stock Market LIVE Updates | Nifty &amp; Sensex Live | Share Market | Business News</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>75</v>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Sale
+Business</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=1_Ih0JYmkjI</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>LIVE 24/7 Domains For Sale | Premium Domain Marketplace</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>75</v>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Sale
+Business</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=fQOMRgEHsEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>kids wear stitched pattu lehenga collection best sale 🥳#9100831197</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>75</v>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Sale
+Business</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=YJLWz2MvYIQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>24/7 UAE Business &amp; Real Estate Hub | Expert Interviews &amp; Market Insights | MIRA Business FM</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>75</v>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Sale
+Business</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=61ItflDkggY</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Як відкрити бізнес (БЕЗ КОМАНДИ) по американській системі ONE PERSON BUSINESS</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>75</v>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Sale
+Business</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=SdV7XI6k5WA</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>​🔴 LIVE: Nikum Fashion MEGA SALE continues! Crazy Discounts on Sandals &amp; Clothes!</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>215</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=ge4xLlledOo</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>raksha bandhan special offer and sale</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>160</v>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=n5ZYjNafPJo</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Super Sunday Anghrakha Special Exclusive Clearance Sale!!!!</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>155</v>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Recruiter, HR Manager</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=nk3ED8Yupic</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>🔴 Live Flash Sale Adenium Bunga Tumpuk Dan Karakter (23 Agustus 2026) #rachmannursery #adenium</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>155</v>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=v5bzraFACwU</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Sakshi Suit Collection is live beautiful suit 😍 Sale Sale Sale 😍 #fashion #live #suits #viral #suit</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>150</v>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=OXxaFUZQIBE</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>🔥💃🚀🚛 Shravanam superfast sale 💥beats work, bits 💥offer, live💥ph 7013425271💥 don’t miss✨</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>95</v>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Recruiter, HR Manager</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Recruitment</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=sMII-zb-uto</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>New Winter Stock Beautiful SALE Dresses</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>90</v>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=-fKhPQsLqiw</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>sravanam maha sale</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>90</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=XISDLxC-N4c</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>The Nandlaala Collection is live…Sunday special sale live..Booking no-9871800667</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>90</v>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=JiuDerZU1pw</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>jagdamba collection is live❤️ Sunday sale dhamaka#8641069309</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>90</v>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=psKQLLDaIU0</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>💕MAHA SALE COTTON SUITS FESTIVE SUIT ☎️ 9548364102</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>90</v>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=zN9-uvFyreE</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Sunday special sale 👜👜👜booking no 8860447712</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>90</v>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Qa83F1E8ayY</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>SALE LƯƠNG VỀ</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>90</v>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=ml9AsHQOxrU</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>JADULAN KOLEKSIAN REDY||SALE MINGGU CERIA😍</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>90</v>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=47kmamY4w9g</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>150 గజాల North Facing G+1 House For Sale | Nagaram Near ECIL | Hyderabad House Tour</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>90</v>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=henjzMJylpc</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>CULTE DU DIM 23-08-2026 | SOIS SALE POUR ETRE UN PANNEAU PUBLICITAIRE | Pasteur : Elie KATALAYI</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>90</v>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Sale</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=7JEfohexZ6w</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>BITCOIN FOREX AI ANALYZER DASHBOARD</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>40</v>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Zoq2XKS7N60</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>GOLD XAU Ai Market Analyzer Live</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>40</v>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=3VstsarTbn0</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>POCKET OPTION LIVE TRADING ➜ POCKET OPTION AI TRADING | POCKET OPTION SIGNALS | POCKET OPTION 2026</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>40</v>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=sFWPGZ32mY0</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>AI Live Radio - Music, News, Podcasts, Weather</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>40</v>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=b41eVHUU0mc</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>BINARY OPTIONS LIVE TRADING ➜ QUOTEX TRADING STRATEGY | BINARY TRADING LIVE | AI TRADING LIVE</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>40</v>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=0_KALTqzQzM</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>The Agentic Web Live: Honeybot Observatory &amp; AI Crawler Telemetry</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>40</v>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=9TMftX7BDYI</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Build with AI | Claude Code, OpenClaw, Cursor and more | 24/7 Live</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>40</v>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=8vaOW_2EpLc</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>CAN YOU BUILD AN AI AGENT—or only use one?</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>40</v>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=Ea4MMH_WcoQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Live Gold (XAUUSD) Trading with EA bot | AI-Based Strategy</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>40</v>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=3xD_Di85Gsc</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>My Personal JARVIS AI 🔴 LIVE — Sara v2 Review And Guide | Ethical CodeX</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>40</v>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=3J8wYG3_kpc</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Future Intelligence 24/7 ⚡ Deep Tech Documentaries | AI Longevity Future of Work</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>40</v>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=mycW8FFaX2A</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>This 24/7 AI-Generated TV channel will make you question reality.</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>40</v>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Ai Automation</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Thấy chủ đề này khá thú vị, không biết thực tế triển khai có hay gặp rào cản gì không mọi người? | Góc nhìn rất thực tế. Cho mình hỏi thêm về case study cụ thể ở mảng này được không? | Phần này mình cũng đang quan tâm. Mọi người thường dùng công cụ gì để giải quyết bài toán này?</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr"/>
+      <c r="I204" t="inlineStr"/>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=6xuQnM810Zw</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr"/>
+      <c r="L204" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update database artifacts, log and cache
</commit_message>
<xml_diff>
--- a/data/livestreams.xlsx
+++ b/data/livestreams.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Livestreams" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Livestreams" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O204"/>
+  <dimension ref="A1:O217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9813,15 +9813,343 @@
           <t>YouTube</t>
         </is>
       </c>
-      <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
       <c r="J204" t="inlineStr">
         <is>
           <t>https://youtube.com/watch?v=6xuQnM810Zw</t>
         </is>
       </c>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Delma #32 student charity member</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>90</v>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=VT3j0maWxx4</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Charity Stream every Brilliant = 3$ (Chat votes to where) 🫂💌👽 !ip !elephant !course !discord</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>80</v>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=BZDLqXTYTTU</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>【直播】 2026-08-23 大專新星 - 宏遠(慈善)籃球聯賽 STAR PATH (CHARITY) BASKETBALL LEAGUE APEX巔峰 vs C &amp; W Charity</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>80</v>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=ljMAh-SuciU</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>【直播】 2026-08-23 大專新星 - 宏遠(慈善)籃球聯賽 STAR PATH (CHARITY) BASKETBALL LEAGUE SV vs VC</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>80</v>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=-mmqCNeIIow</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>RIVER NETWORK TV, Church, Charity, DERBYSHIRE Terry &amp; Jill Eckersley</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>80</v>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=hWKwOuAhZVc</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>🔴 LIVE: Adam Littler XI vs Michael Littler XI | Julie Littler Memorial Charity Fixture</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>80</v>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=jaoHESV8-RQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>kalayami cultural charitable trust is live</t>
+        </is>
+      </c>
+      <c r="B211" t="n">
+        <v>58</v>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=CaNr-dsHJt8</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Power And Authority(Part 9) - Christingle Fellowship Centre</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>51</v>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=GvXLs4slBcM</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Morning Service - 23 August 2026 Bon Accord Free Church</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>49</v>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=mNrDxsjQ_1g</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Unity &amp; Diversity Culture Service - Pauline Dawkins - Livestream - 23.08.2026</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>44</v>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=RJBVodYmtdQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>[SUN. 23RD-AUG-2026AM] SUNDAY MORNING SERVICE</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>39</v>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=oX8gp-vPlQo</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Welcome to our morning worship on Sunday 23rd August 2026.</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>35</v>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=SJdGhQYHiXI</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Back to school sunday 16th August 2026</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>33</v>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr"/>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr"/>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr"/>
+      <c r="I217" t="inlineStr"/>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>https://youtube.com/watch?v=1hkGi2ISc5g</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr"/>
+      <c r="L217" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>